<commit_message>
att centenario do sul 2026
</commit_message>
<xml_diff>
--- a/data/dados.xlsx
+++ b/data/dados.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\reajuste\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E7E25C7-86AE-4EA0-A768-892F8D58BBF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A862386-40AA-46FE-BAB1-6CA486A26AE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="15585" xr2:uid="{BE2A1F3B-6535-41F1-9783-CEB15E5262F6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{BE2A1F3B-6535-41F1-9783-CEB15E5262F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="81">
   <si>
     <t>Cafeara</t>
   </si>
@@ -277,6 +277,9 @@
   </si>
   <si>
     <t>Populacao</t>
+  </si>
+  <si>
+    <t>https://www.diariomunicipal.com.br/amp/materia/732EB9FD/f71481bba070e988d1c4ee95c9001e57f71481bba070e988d1c4ee95c9001e57</t>
   </si>
 </sst>
 </file>
@@ -733,7 +736,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95A9F774-A2B7-43E0-89BB-A01627A8B05C}">
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:G74"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.42578125" style="3" bestFit="1" customWidth="1"/>
@@ -1157,15 +1160,15 @@
       <c r="D26" s="14"/>
       <c r="E26" s="14"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>52</v>
       </c>
       <c r="B27" s="5">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C27" s="7">
-        <v>0.05</v>
+        <v>4.2599999999999999E-2</v>
       </c>
       <c r="D27" s="14">
         <v>4105102</v>
@@ -1173,8 +1176,8 @@
       <c r="E27" s="14">
         <v>10903</v>
       </c>
-      <c r="F27" s="3" t="s">
-        <v>22</v>
+      <c r="F27" s="10" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
@@ -1182,7 +1185,7 @@
         <v>52</v>
       </c>
       <c r="B28" s="5">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C28" s="7">
         <v>0.05</v>
@@ -1194,7 +1197,7 @@
         <v>10903</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
@@ -1202,10 +1205,10 @@
         <v>52</v>
       </c>
       <c r="B29" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C29" s="7">
-        <v>5.9299999999999999E-2</v>
+        <v>0.05</v>
       </c>
       <c r="D29" s="14">
         <v>4105102</v>
@@ -1214,7 +1217,7 @@
         <v>10903</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
@@ -1222,10 +1225,10 @@
         <v>52</v>
       </c>
       <c r="B30" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C30" s="7">
-        <v>0.1016</v>
+        <v>5.9299999999999999E-2</v>
       </c>
       <c r="D30" s="14">
         <v>4105102</v>
@@ -1234,7 +1237,7 @@
         <v>10903</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -1242,10 +1245,10 @@
         <v>52</v>
       </c>
       <c r="B31" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C31" s="7">
-        <v>4.5199999999999997E-2</v>
+        <v>0.1016</v>
       </c>
       <c r="D31" s="14">
         <v>4105102</v>
@@ -1254,7 +1257,7 @@
         <v>10903</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
@@ -1262,10 +1265,10 @@
         <v>52</v>
       </c>
       <c r="B32" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C32" s="7">
-        <v>4.48E-2</v>
+        <v>4.5199999999999997E-2</v>
       </c>
       <c r="D32" s="14">
         <v>4105102</v>
@@ -1274,40 +1277,40 @@
         <v>10903</v>
       </c>
       <c r="F32" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A33" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="5">
+        <v>2020</v>
+      </c>
+      <c r="C33" s="7">
+        <v>4.48E-2</v>
+      </c>
+      <c r="D33" s="14">
+        <v>4105102</v>
+      </c>
+      <c r="E33" s="14">
+        <v>10903</v>
+      </c>
+      <c r="F33" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C33" s="7"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-    </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A34" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B34" s="5">
-        <v>2025</v>
-      </c>
-      <c r="C34" s="7">
-        <v>0.05</v>
-      </c>
-      <c r="D34" s="14">
-        <v>4113809</v>
-      </c>
-      <c r="E34" s="14">
-        <v>4929</v>
-      </c>
-      <c r="F34" s="3" t="s">
-        <v>30</v>
-      </c>
+      <c r="C34" s="7"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
         <v>51</v>
       </c>
       <c r="B35" s="5">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C35" s="7">
         <v>0.05</v>
@@ -1319,7 +1322,7 @@
         <v>4929</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
@@ -1327,10 +1330,10 @@
         <v>51</v>
       </c>
       <c r="B36" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C36" s="7">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
       <c r="D36" s="14">
         <v>4113809</v>
@@ -1339,7 +1342,7 @@
         <v>4929</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
@@ -1347,10 +1350,10 @@
         <v>51</v>
       </c>
       <c r="B37" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C37" s="7">
-        <v>5.45E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="D37" s="14">
         <v>4113809</v>
@@ -1359,7 +1362,7 @@
         <v>4929</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
@@ -1370,7 +1373,7 @@
         <v>2022</v>
       </c>
       <c r="C38" s="7">
-        <v>0.1016</v>
+        <v>5.45E-2</v>
       </c>
       <c r="D38" s="14">
         <v>4113809</v>
@@ -1379,7 +1382,7 @@
         <v>4929</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
@@ -1387,14 +1390,19 @@
         <v>51</v>
       </c>
       <c r="B39" s="5">
-        <v>2021</v>
-      </c>
-      <c r="C39" s="7"/>
+        <v>2022</v>
+      </c>
+      <c r="C39" s="7">
+        <v>0.1016</v>
+      </c>
       <c r="D39" s="14">
         <v>4113809</v>
       </c>
       <c r="E39" s="14">
         <v>4929</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
@@ -1402,52 +1410,47 @@
         <v>51</v>
       </c>
       <c r="B40" s="5">
-        <v>2020</v>
-      </c>
-      <c r="C40" s="7">
-        <v>4.48E-2</v>
-      </c>
+        <v>2021</v>
+      </c>
+      <c r="C40" s="7"/>
       <c r="D40" s="14">
         <v>4113809</v>
       </c>
       <c r="E40" s="14">
         <v>4929</v>
       </c>
-      <c r="F40" s="3" t="s">
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A41" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B41" s="5">
+        <v>2020</v>
+      </c>
+      <c r="C41" s="7">
+        <v>4.48E-2</v>
+      </c>
+      <c r="D41" s="14">
+        <v>4113809</v>
+      </c>
+      <c r="E41" s="14">
+        <v>4929</v>
+      </c>
+      <c r="F41" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C41" s="7"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-    </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A42" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B42" s="5">
-        <v>2025</v>
-      </c>
-      <c r="C42" s="7">
-        <v>0.05</v>
-      </c>
-      <c r="D42" s="14">
-        <v>4111902</v>
-      </c>
-      <c r="E42" s="14">
-        <v>15908</v>
-      </c>
-      <c r="F42" s="3" t="s">
-        <v>35</v>
-      </c>
+      <c r="C42" s="7"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
         <v>50</v>
       </c>
       <c r="B43" s="5">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C43" s="7">
         <v>0.05</v>
@@ -1459,7 +1462,7 @@
         <v>15908</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
@@ -1467,10 +1470,10 @@
         <v>50</v>
       </c>
       <c r="B44" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C44" s="7">
-        <v>0.14949999999999999</v>
+        <v>0.05</v>
       </c>
       <c r="D44" s="14">
         <v>4111902</v>
@@ -1479,7 +1482,7 @@
         <v>15908</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
@@ -1487,10 +1490,10 @@
         <v>50</v>
       </c>
       <c r="B45" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C45" s="7">
-        <v>0.15</v>
+        <v>0.14949999999999999</v>
       </c>
       <c r="D45" s="14">
         <v>4111902</v>
@@ -1499,7 +1502,7 @@
         <v>15908</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
@@ -1507,10 +1510,10 @@
         <v>50</v>
       </c>
       <c r="B46" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C46" s="7">
-        <v>5.5300000000000002E-2</v>
+        <v>0.15</v>
       </c>
       <c r="D46" s="14">
         <v>4111902</v>
@@ -1519,7 +1522,7 @@
         <v>15908</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
@@ -1527,10 +1530,10 @@
         <v>50</v>
       </c>
       <c r="B47" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C47" s="7">
-        <v>2.2499999999999999E-2</v>
+        <v>5.5300000000000002E-2</v>
       </c>
       <c r="D47" s="14">
         <v>4111902</v>
@@ -1539,43 +1542,43 @@
         <v>15908</v>
       </c>
       <c r="F47" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A48" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B48" s="5">
+        <v>2020</v>
+      </c>
+      <c r="C48" s="7">
+        <v>2.2499999999999999E-2</v>
+      </c>
+      <c r="D48" s="14">
+        <v>4111902</v>
+      </c>
+      <c r="E48" s="14">
+        <v>15908</v>
+      </c>
+      <c r="F48" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C48" s="7"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
-    </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A49" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B49" s="5">
-        <v>2025</v>
-      </c>
-      <c r="C49" s="7">
-        <v>4.8300000000000003E-2</v>
-      </c>
-      <c r="D49" s="14">
-        <v>4120507</v>
-      </c>
-      <c r="E49" s="14">
-        <v>10064</v>
-      </c>
-      <c r="F49" s="3" t="s">
-        <v>46</v>
-      </c>
+      <c r="C49" s="7"/>
+      <c r="D49" s="14"/>
+      <c r="E49" s="14"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
         <v>43</v>
       </c>
       <c r="B50" s="5">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C50" s="7">
-        <v>0.11460000000000001</v>
+        <v>4.8300000000000003E-2</v>
       </c>
       <c r="D50" s="14">
         <v>4120507</v>
@@ -1584,7 +1587,7 @@
         <v>10064</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.2">
@@ -1592,10 +1595,10 @@
         <v>43</v>
       </c>
       <c r="B51" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C51" s="7">
-        <v>0.1263</v>
+        <v>0.11460000000000001</v>
       </c>
       <c r="D51" s="14">
         <v>4120507</v>
@@ -1604,7 +1607,7 @@
         <v>10064</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.2">
@@ -1612,10 +1615,10 @@
         <v>43</v>
       </c>
       <c r="B52" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C52" s="7">
-        <v>0.15</v>
+        <v>0.1263</v>
       </c>
       <c r="D52" s="14">
         <v>4120507</v>
@@ -1624,7 +1627,7 @@
         <v>10064</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
@@ -1632,10 +1635,10 @@
         <v>43</v>
       </c>
       <c r="B53" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C53" s="7">
-        <v>4.5199999999999997E-2</v>
+        <v>0.15</v>
       </c>
       <c r="D53" s="14">
         <v>4120507</v>
@@ -1644,7 +1647,7 @@
         <v>10064</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
@@ -1652,10 +1655,10 @@
         <v>43</v>
       </c>
       <c r="B54" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C54" s="7">
-        <v>7.3178999999999994E-2</v>
+        <v>4.5199999999999997E-2</v>
       </c>
       <c r="D54" s="14">
         <v>4120507</v>
@@ -1664,42 +1667,42 @@
         <v>10064</v>
       </c>
       <c r="F54" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A55" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B55" s="5">
+        <v>2020</v>
+      </c>
+      <c r="C55" s="7">
+        <v>7.3178999999999994E-2</v>
+      </c>
+      <c r="D55" s="14">
+        <v>4120507</v>
+      </c>
+      <c r="E55" s="14">
+        <v>10064</v>
+      </c>
+      <c r="F55" s="3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D55" s="14"/>
-      <c r="E55" s="14"/>
-    </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A56" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B56" s="5">
-        <v>2025</v>
-      </c>
-      <c r="C56" s="17">
-        <v>4.8300000000000003E-2</v>
-      </c>
-      <c r="D56" s="14">
-        <v>4120333</v>
-      </c>
-      <c r="E56" s="14">
-        <v>3816</v>
-      </c>
-      <c r="F56" s="3" t="s">
-        <v>56</v>
-      </c>
+      <c r="D56" s="14"/>
+      <c r="E56" s="14"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
         <v>54</v>
       </c>
       <c r="B57" s="5">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C57" s="17">
-        <v>4.6199999999999998E-2</v>
+        <v>4.8300000000000003E-2</v>
       </c>
       <c r="D57" s="14">
         <v>4120333</v>
@@ -1708,7 +1711,7 @@
         <v>3816</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.2">
@@ -1716,10 +1719,10 @@
         <v>54</v>
       </c>
       <c r="B58" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C58" s="17">
-        <v>5.9299999999999999E-2</v>
+        <v>4.6199999999999998E-2</v>
       </c>
       <c r="D58" s="14">
         <v>4120333</v>
@@ -1728,7 +1731,7 @@
         <v>3816</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.2">
@@ -1736,10 +1739,10 @@
         <v>54</v>
       </c>
       <c r="B59" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C59" s="17">
-        <v>0.1</v>
+        <v>5.9299999999999999E-2</v>
       </c>
       <c r="D59" s="14">
         <v>4120333</v>
@@ -1748,7 +1751,7 @@
         <v>3816</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.2">
@@ -1756,10 +1759,10 @@
         <v>54</v>
       </c>
       <c r="B60" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C60" s="17">
-        <v>4.5199999999999997E-2</v>
+        <v>0.1</v>
       </c>
       <c r="D60" s="14">
         <v>4120333</v>
@@ -1768,7 +1771,7 @@
         <v>3816</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.2">
@@ -1776,10 +1779,10 @@
         <v>54</v>
       </c>
       <c r="B61" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C61" s="17">
-        <v>4.3099999999999999E-2</v>
+        <v>4.5199999999999997E-2</v>
       </c>
       <c r="D61" s="14">
         <v>4120333</v>
@@ -1788,41 +1791,41 @@
         <v>3816</v>
       </c>
       <c r="F61" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A62" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B62" s="5">
+        <v>2020</v>
+      </c>
+      <c r="C62" s="17">
+        <v>4.3099999999999999E-2</v>
+      </c>
+      <c r="D62" s="14">
+        <v>4120333</v>
+      </c>
+      <c r="E62" s="14">
+        <v>3816</v>
+      </c>
+      <c r="F62" s="3" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E62" s="14"/>
-    </row>
-    <row r="63" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A63" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B63" s="5">
-        <v>2025</v>
-      </c>
-      <c r="C63" s="7">
-        <v>0.05</v>
-      </c>
-      <c r="D63" s="14">
-        <v>4123402</v>
-      </c>
-      <c r="E63" s="14">
-        <v>11730</v>
-      </c>
-      <c r="F63" s="10" t="s">
-        <v>71</v>
-      </c>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E63" s="14"/>
     </row>
     <row r="64" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
         <v>70</v>
       </c>
       <c r="B64" s="5">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C64" s="7">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="D64" s="14">
         <v>4123402</v>
@@ -1831,7 +1834,7 @@
         <v>11730</v>
       </c>
       <c r="F64" s="10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="65" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
@@ -1839,10 +1842,10 @@
         <v>70</v>
       </c>
       <c r="B65" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C65" s="7">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="D65" s="14">
         <v>4123402</v>
@@ -1851,7 +1854,7 @@
         <v>11730</v>
       </c>
       <c r="F65" s="10" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="66" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
@@ -1859,10 +1862,10 @@
         <v>70</v>
       </c>
       <c r="B66" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C66" s="7">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="D66" s="14">
         <v>4123402</v>
@@ -1871,7 +1874,7 @@
         <v>11730</v>
       </c>
       <c r="F66" s="10" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="67" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
@@ -1891,7 +1894,7 @@
         <v>11730</v>
       </c>
       <c r="F67" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="68" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
@@ -1899,10 +1902,10 @@
         <v>70</v>
       </c>
       <c r="B68" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C68" s="7">
-        <v>4.5199999999999997E-2</v>
+        <v>0.15</v>
       </c>
       <c r="D68" s="14">
         <v>4123402</v>
@@ -1911,7 +1914,7 @@
         <v>11730</v>
       </c>
       <c r="F68" s="10" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="69" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
@@ -1919,10 +1922,10 @@
         <v>70</v>
       </c>
       <c r="B69" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C69" s="7">
-        <v>4.3099999999999999E-2</v>
+        <v>4.5199999999999997E-2</v>
       </c>
       <c r="D69" s="14">
         <v>4123402</v>
@@ -1931,11 +1934,28 @@
         <v>11730</v>
       </c>
       <c r="F69" s="10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="A70" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B70" s="5">
+        <v>2020</v>
+      </c>
+      <c r="C70" s="7">
+        <v>4.3099999999999999E-2</v>
+      </c>
+      <c r="D70" s="14">
+        <v>4123402</v>
+      </c>
+      <c r="E70" s="14">
+        <v>11730</v>
+      </c>
+      <c r="F70" s="10" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E70" s="14"/>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="E71" s="14"/>
@@ -1945,6 +1965,9 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="E73" s="14"/>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E74" s="14"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1962,49 +1985,50 @@
     <hyperlink ref="F23" r:id="rId12" display="https://leis.org/municipais/pr/cafeara/lei/lei-ordinaria/2022/587/lei-ordinaria-n-587-2022-autoriza-o-executivo-municipal-a-conceder-recomposicao-geral-anual-aos-servidores-publicos-municipais-e-agentes-politicos-do-poder-executivo-municipal-de-cafeara-e-da-outras-providencias?termo=RECOMPOSI%C3%87%C3%83O%20GERAL%20ANUAL" xr:uid="{1B38F967-CA98-456B-9E39-53D8B29C2593}"/>
     <hyperlink ref="F24" r:id="rId13" display="https://leis.org/municipais/pr/cafeara/lei/lei-ordinaria/2021/563/lei-ordinaria-n-563-2021-autoriza-o-executivo-municipal-a-conceder-recomposicao-geral-anual-aos-servidores-publicos-municipais-e-agentes-politicos-do-poder-executivo-municipal-de-cafeara-e-da-outras-providencias?termo=RECOMPOSI%C3%87%C3%83O%20GERAL%20ANUAL" xr:uid="{2F2E9EFC-04E5-4D6C-ADAE-3D1C1FE4D8C2}"/>
     <hyperlink ref="F25" r:id="rId14" display="https://leis.org/municipais/pr/cafeara/lei/lei-ordinaria/2020/542/lei-ordinaria-n-542-2020-autoriza-o-executivo-municipal-a-conceder-recomposicao-geral-anual-aos-servidores-publicos-municipais-e-agentes-politicos-do-poder-executivo-municipal-de-cafeara-e-revisao-salarial-aos-servidores-publicos-municipais-e-da-outras-providencias?termo=RECOMPOSI%C3%87%C3%83O%20GERAL%20ANUAL" xr:uid="{CE150FB9-81B7-4D95-A8CF-6EF4FEC69817}"/>
-    <hyperlink ref="F27" r:id="rId15" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2025/325/3248/lei-ordinaria-n-3248-2025-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-com-excecao-dos-subsidios-dos-agentes-politicos?q=reajuste" xr:uid="{14532045-718C-41E1-8B54-50EFD37FBDB7}"/>
-    <hyperlink ref="F28" r:id="rId16" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2024/322/3211/lei-ordinaria-n-3211-2024-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-inclusive-sobre-os-subsidios-dos-agentes-politicos?q=reajuste" xr:uid="{38AE6B04-78B2-4EB9-9571-DB2D521C73B5}"/>
-    <hyperlink ref="F29" r:id="rId17" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2023/317/3170/lei-ordinaria-n-3170-2023-autoriza-a-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-inclusive-sobre-os-subsidios-dos-agentes-politicos?q=reajuste" xr:uid="{4CF69429-E3A8-42D6-85E9-C1B4DF636DEA}"/>
-    <hyperlink ref="F30" r:id="rId18" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2022/314/3132/lei-ordinaria-n-3132-2022-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-inclusive-sobre-os-subsidios-dos-agentes-politicos?q=reajuste" xr:uid="{55BFE9D4-B84C-4424-B8D7-86FC64A9AB3E}"/>
-    <hyperlink ref="F31" r:id="rId19" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2021/310/3097/lei-ordinaria-n-3097-2021-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao?q=reajuste" xr:uid="{87876156-98C2-4000-91CE-7C8AD0B3476E}"/>
-    <hyperlink ref="F32" r:id="rId20" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2020/305/3045/lei-ordinaria-n-3045-2020-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-inclusive-sobre-os-subsidios-dos-agentes-politicos-bem-como-adequa-o-salario-dos-servidores-do-quadro-do-magisterio-publico-municipal-ao-piso-salarial-profissional-nacional?q=reajuste" xr:uid="{DF65B76A-65AA-4C35-A537-F477C0AB6BF4}"/>
+    <hyperlink ref="F28" r:id="rId15" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2025/325/3248/lei-ordinaria-n-3248-2025-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-com-excecao-dos-subsidios-dos-agentes-politicos?q=reajuste" xr:uid="{14532045-718C-41E1-8B54-50EFD37FBDB7}"/>
+    <hyperlink ref="F29" r:id="rId16" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2024/322/3211/lei-ordinaria-n-3211-2024-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-inclusive-sobre-os-subsidios-dos-agentes-politicos?q=reajuste" xr:uid="{38AE6B04-78B2-4EB9-9571-DB2D521C73B5}"/>
+    <hyperlink ref="F30" r:id="rId17" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2023/317/3170/lei-ordinaria-n-3170-2023-autoriza-a-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-inclusive-sobre-os-subsidios-dos-agentes-politicos?q=reajuste" xr:uid="{4CF69429-E3A8-42D6-85E9-C1B4DF636DEA}"/>
+    <hyperlink ref="F31" r:id="rId18" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2022/314/3132/lei-ordinaria-n-3132-2022-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-inclusive-sobre-os-subsidios-dos-agentes-politicos?q=reajuste" xr:uid="{55BFE9D4-B84C-4424-B8D7-86FC64A9AB3E}"/>
+    <hyperlink ref="F32" r:id="rId19" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2021/310/3097/lei-ordinaria-n-3097-2021-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao?q=reajuste" xr:uid="{87876156-98C2-4000-91CE-7C8AD0B3476E}"/>
+    <hyperlink ref="F33" r:id="rId20" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2020/305/3045/lei-ordinaria-n-3045-2020-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-inclusive-sobre-os-subsidios-dos-agentes-politicos-bem-como-adequa-o-salario-dos-servidores-do-quadro-do-magisterio-publico-municipal-ao-piso-salarial-profissional-nacional?q=reajuste" xr:uid="{DF65B76A-65AA-4C35-A537-F477C0AB6BF4}"/>
     <hyperlink ref="G18" r:id="rId21" xr:uid="{EC4616F6-7680-425A-9B5B-FA1377623831}"/>
     <hyperlink ref="F10" r:id="rId22" xr:uid="{5B0B0D6A-84BF-4334-B8E3-04EFE33A5016}"/>
     <hyperlink ref="F2" r:id="rId23" xr:uid="{5300EFF3-C77D-4044-9FEE-10FEE221CCA5}"/>
-    <hyperlink ref="F34" r:id="rId24" xr:uid="{0198FF07-6ABC-4FE0-BC94-9626A092EF1E}"/>
-    <hyperlink ref="F35" r:id="rId25" xr:uid="{9B9DADFC-147D-439F-A89B-8D7EC2EFFA45}"/>
-    <hyperlink ref="F36" r:id="rId26" xr:uid="{7B4312A5-B4D6-48C3-9967-D4A547A0F189}"/>
-    <hyperlink ref="F40" r:id="rId27" xr:uid="{B555F1DF-7AE0-4CE3-A746-A72DB71A3814}"/>
-    <hyperlink ref="F42" r:id="rId28" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2025/1/3/lei-ordinaria-n-3-2025-concede-recomposicao-e-reajuste-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{79AF655C-919A-4B59-8D63-6E9B71A0DFD8}"/>
-    <hyperlink ref="F43" r:id="rId29" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2024/1/6/lei-ordinaria-n-6-2024-concede-recomposicao-e-reajuste-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-e-recomposicao-inflacionaria-aos-agentes-politicos-do-poder-executivo-prefeito-vice-prefeito-e-secretarios-municipais-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{28DF2AEC-02FD-4904-92E4-8F1A46B7C53A}"/>
-    <hyperlink ref="F44" r:id="rId30" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2023/1/3/lei-ordinaria-n-3-2023-concede-recomposicao-e-reajuste-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-e-recomposicao-inflacionaria-aos-agentes-politicos-do-poder-executivo-prefeito-vice-prefeito-e-secretarios-municipais-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{D52BDBF7-13A5-4A80-A127-116B587657FB}"/>
-    <hyperlink ref="F45" r:id="rId31" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2022/1/5/lei-ordinaria-n-5-2022-concede-recomposicao-e-reajuste-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{3E75ABFE-1194-4B2F-AF68-D20DEC412ED8}"/>
-    <hyperlink ref="F46" r:id="rId32" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2021/1/5/lei-ordinaria-n-5-2021-concede-recomposicao-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{4FC8FEEE-0401-4369-8921-ED4B51F5562D}"/>
-    <hyperlink ref="F47" r:id="rId33" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2020/2/11/lei-ordinaria-n-11-2020-concede-recomposicao-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-e-ao-prefeito-vice-prefeito-e-secretarios-municipais-desta-municipalidade-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{4D8E764E-22B9-4B1F-A195-598C7E088B03}"/>
-    <hyperlink ref="F51" r:id="rId34" xr:uid="{469628B4-8B6D-46C9-A62E-832B5D06C62E}"/>
-    <hyperlink ref="F54" r:id="rId35" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2020/74/739/lei-ordinaria-n-739-2020-dispoe-sobre-a-revisao-geral-anual-do-subsidio-do-prefeito-vice-prefeito-vereadores-secretarios-as-municipais-e-remuneracao-do-s-servidor-es-comissionados-e-estatutario-do-poder-legislativo-do-municipio-de-primeiro-de-maio-e-da-outras-providencias?q=salarial%20" xr:uid="{8F367E47-ABB7-4AAB-A611-4BB40BDA61A3}"/>
-    <hyperlink ref="F49" r:id="rId36" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2025/97/970/lei-ordinaria-n-970-2025-dispoe-sobre-a-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-municipais-de-primeiro-de-maio-e-da-outras-providencias?q=revis%E3o%20geral%20anual%20" xr:uid="{9C1E9D0B-D3E4-4ECB-928C-3AB9384788C0}"/>
-    <hyperlink ref="F50" r:id="rId37" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2024/94/934/lei-ordinaria-n-934-2024-dispoe-sobre-a-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-municipais-de-primeiro-de-maio-e-da-outras-providencias?q=revis%E3o%20geral%20anual%20" xr:uid="{AF964D4D-7701-48C8-898F-A6225D73AC79}"/>
-    <hyperlink ref="F52" r:id="rId38" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2022/80/800/lei-ordinaria-n-800-2022-dispoe-sobre-a-revisao-geral-anual-do-subsidio-do-prefeito-vice-prefeito-vereadores-secretarios-as-municipais-e-remuneracao-do-s-servidor-es-comissionados-e-estatutario-do-poder-legislativo-do-municipio-de-primeiro-de-maio-e-da-outras-providencias?q=revis%E3o%20geral%20anual%20" xr:uid="{98F545B3-8D3D-44B1-AB35-4AC2759963EB}"/>
-    <hyperlink ref="F53" r:id="rId39" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2021/77/770/lei-ordinaria-n-770-2021-dispoe-sobre-a-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-municipais-de-primeiro-de-maio-e-da-outras-providencias?q=revis%E3o%20geral%20anual%20" xr:uid="{C52DDB23-FB88-489B-BD74-E79A0801ADF5}"/>
-    <hyperlink ref="F38" r:id="rId40" xr:uid="{878A7E66-55B4-4DAF-8A75-A1CF624BBEC7}"/>
-    <hyperlink ref="F37" r:id="rId41" xr:uid="{47F34AB3-0A0A-412F-8FE1-03EF5CACC9CA}"/>
-    <hyperlink ref="F59" r:id="rId42" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-complementar/2022/59/583/lei-complementar-n-583-2022-dispoe-sobre-aumento-salarial-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=aumento%20salarial" xr:uid="{9456DAAA-0A8A-485D-A402-82BED62E4A97}"/>
-    <hyperlink ref="F56" r:id="rId43" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2025/63/630/lei-ordinaria-n-630-2025-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{64BC75ED-1964-4204-BAFA-49F3A4083336}"/>
-    <hyperlink ref="F57" r:id="rId44" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2024/62/614/lei-ordinaria-n-614-2024-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{0661ED8C-7E04-4235-BDA6-165CAA2FD04B}"/>
-    <hyperlink ref="F58" r:id="rId45" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2023/59/588/lei-ordinaria-n-588-2023-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{4A341ABB-8BE7-4A6E-B4C1-532DBB4378D2}"/>
-    <hyperlink ref="F60" r:id="rId46" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2021/54/534/lei-ordinaria-n-534-2021-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{95B75048-0C9A-47CB-8A73-3D8052953EA1}"/>
-    <hyperlink ref="F61" r:id="rId47" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2020/52/516/lei-ordinaria-n-516-2020-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{46529EB6-AC15-4D01-B558-28DB00531128}"/>
-    <hyperlink ref="F63" r:id="rId48" xr:uid="{EE42FF6B-39FA-43BE-8F7C-A56762A03BE5}"/>
-    <hyperlink ref="F64" r:id="rId49" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2024/232/2320/lei-ordinaria-n-2320-2024-autoriza-revisao-geral-da-remuneracao-e-os-subsidios-dos-servidores-publicos-e-agentes-politicos-dos-poderes-executivo-e-legislativo-do-municipio-nos-termos-do-artigo-7-caput-iv-e-o-do-artigo-39-3-da-constituicao-federal-extensivo-aos-conselheiros-tutelares-e-aos-proventos-dos-inativos-e-pensionistas?q=Revis%C3%A3o+geraL" xr:uid="{4F7B275E-5955-4B1B-94E6-A35B6D80FEE2}"/>
-    <hyperlink ref="F68" r:id="rId50" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2021/218/2180/lei-ordinaria-n-2180-2021-suspende-os-efeitos-da-lei-municipal-n-2147-2021-que-autoriza-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-e-da-outras-providencias?q=Revis%E3o%20geraL" xr:uid="{EB57F7DB-CDEF-4A7C-9E25-23B1204FA785}"/>
-    <hyperlink ref="F69" r:id="rId51" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2020/211/2107/lei-ordinaria-n-2107-2020-autoriza-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-a-aplicacao-do-artigo-7-inciso-iv-e-art-39-3-da-constituicao-federal-a-remuneracao-dos-servidores-publicos-o-reajuste-dos-proventos-dos-inativos-e-pensionistas-a-recomposicao-dos-subsidios-dos-agentes-politicos-e-fixa-os-pisos-nacionais-minimos-para-os-integrantes-do-magisterio-municipal-11739-2008-e-da-outras-providencias?q=Revis%E3o%20geraL" xr:uid="{924B3E23-6A28-4DA7-BF55-853A35BD0084}"/>
-    <hyperlink ref="F66" r:id="rId52" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2021/220/2198/lei-ordinaria-n-2198-2021-autoriza-revisao-geral-da-remuneracao-dos-servidores-publicos-autoriza-a-aplicacao-do-artigo-7-caput-iv-e-o-do-artigo-39-3-da-constituicao-federal-a-remuneracao-dos-servidores-publicos-e-autoriza-o-reajuste-dos-proventos-dos-inativos-e-pensionistas?q=2.198" xr:uid="{D3688214-1F73-4C24-86E5-7E744B395889}"/>
-    <hyperlink ref="F67" r:id="rId53" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2021/220/2197/lei-ordinaria-n-2197-2021-autoriza-revisao-geral-da-remuneracao-dos-servidores-publicos-autoriza-a-aplicacao-do-artigo-7-caput-iv-e-o-do-artigo-39-3-da-constituicao-federal-a-remuneracao-dos-servidores-publicos-e-autoriza-o-reajuste-dos-proventos-dos-inativos-e-pensionistas?q=2.197" xr:uid="{824C9DCD-78D8-43FD-8DB5-0E165BC5D312}"/>
-    <hyperlink ref="F65" r:id="rId54" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2023/226/2251/lei-ordinaria-n-2251-2023-autoriza-revisao-geral-da-remuneracao-e-os-subsidios-dos-servidores-publicos-e-agentes-politicos-dos-poderes-executivo-e-legislativo-do-municipio-nos-termos-do-artigo-7-caput-iv-e-o-do-artigo-39-3-da-constituicao-federal-extensivo-aos-conselheiros-tutelares-e-aos-proventos-dos-inativos-e-pensionistas?q=Autoriza%20revis%E3o%20geral%20da%20remunera%E7%E3o" xr:uid="{7E99F84F-40DA-489D-BFB8-FC337539CA92}"/>
+    <hyperlink ref="F35" r:id="rId24" xr:uid="{0198FF07-6ABC-4FE0-BC94-9626A092EF1E}"/>
+    <hyperlink ref="F36" r:id="rId25" xr:uid="{9B9DADFC-147D-439F-A89B-8D7EC2EFFA45}"/>
+    <hyperlink ref="F37" r:id="rId26" xr:uid="{7B4312A5-B4D6-48C3-9967-D4A547A0F189}"/>
+    <hyperlink ref="F41" r:id="rId27" xr:uid="{B555F1DF-7AE0-4CE3-A746-A72DB71A3814}"/>
+    <hyperlink ref="F43" r:id="rId28" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2025/1/3/lei-ordinaria-n-3-2025-concede-recomposicao-e-reajuste-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{79AF655C-919A-4B59-8D63-6E9B71A0DFD8}"/>
+    <hyperlink ref="F44" r:id="rId29" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2024/1/6/lei-ordinaria-n-6-2024-concede-recomposicao-e-reajuste-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-e-recomposicao-inflacionaria-aos-agentes-politicos-do-poder-executivo-prefeito-vice-prefeito-e-secretarios-municipais-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{28DF2AEC-02FD-4904-92E4-8F1A46B7C53A}"/>
+    <hyperlink ref="F45" r:id="rId30" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2023/1/3/lei-ordinaria-n-3-2023-concede-recomposicao-e-reajuste-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-e-recomposicao-inflacionaria-aos-agentes-politicos-do-poder-executivo-prefeito-vice-prefeito-e-secretarios-municipais-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{D52BDBF7-13A5-4A80-A127-116B587657FB}"/>
+    <hyperlink ref="F46" r:id="rId31" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2022/1/5/lei-ordinaria-n-5-2022-concede-recomposicao-e-reajuste-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{3E75ABFE-1194-4B2F-AF68-D20DEC412ED8}"/>
+    <hyperlink ref="F47" r:id="rId32" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2021/1/5/lei-ordinaria-n-5-2021-concede-recomposicao-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{4FC8FEEE-0401-4369-8921-ED4B51F5562D}"/>
+    <hyperlink ref="F48" r:id="rId33" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2020/2/11/lei-ordinaria-n-11-2020-concede-recomposicao-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-e-ao-prefeito-vice-prefeito-e-secretarios-municipais-desta-municipalidade-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{4D8E764E-22B9-4B1F-A195-598C7E088B03}"/>
+    <hyperlink ref="F52" r:id="rId34" xr:uid="{469628B4-8B6D-46C9-A62E-832B5D06C62E}"/>
+    <hyperlink ref="F55" r:id="rId35" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2020/74/739/lei-ordinaria-n-739-2020-dispoe-sobre-a-revisao-geral-anual-do-subsidio-do-prefeito-vice-prefeito-vereadores-secretarios-as-municipais-e-remuneracao-do-s-servidor-es-comissionados-e-estatutario-do-poder-legislativo-do-municipio-de-primeiro-de-maio-e-da-outras-providencias?q=salarial%20" xr:uid="{8F367E47-ABB7-4AAB-A611-4BB40BDA61A3}"/>
+    <hyperlink ref="F50" r:id="rId36" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2025/97/970/lei-ordinaria-n-970-2025-dispoe-sobre-a-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-municipais-de-primeiro-de-maio-e-da-outras-providencias?q=revis%E3o%20geral%20anual%20" xr:uid="{9C1E9D0B-D3E4-4ECB-928C-3AB9384788C0}"/>
+    <hyperlink ref="F51" r:id="rId37" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2024/94/934/lei-ordinaria-n-934-2024-dispoe-sobre-a-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-municipais-de-primeiro-de-maio-e-da-outras-providencias?q=revis%E3o%20geral%20anual%20" xr:uid="{AF964D4D-7701-48C8-898F-A6225D73AC79}"/>
+    <hyperlink ref="F53" r:id="rId38" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2022/80/800/lei-ordinaria-n-800-2022-dispoe-sobre-a-revisao-geral-anual-do-subsidio-do-prefeito-vice-prefeito-vereadores-secretarios-as-municipais-e-remuneracao-do-s-servidor-es-comissionados-e-estatutario-do-poder-legislativo-do-municipio-de-primeiro-de-maio-e-da-outras-providencias?q=revis%E3o%20geral%20anual%20" xr:uid="{98F545B3-8D3D-44B1-AB35-4AC2759963EB}"/>
+    <hyperlink ref="F54" r:id="rId39" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2021/77/770/lei-ordinaria-n-770-2021-dispoe-sobre-a-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-municipais-de-primeiro-de-maio-e-da-outras-providencias?q=revis%E3o%20geral%20anual%20" xr:uid="{C52DDB23-FB88-489B-BD74-E79A0801ADF5}"/>
+    <hyperlink ref="F39" r:id="rId40" xr:uid="{878A7E66-55B4-4DAF-8A75-A1CF624BBEC7}"/>
+    <hyperlink ref="F38" r:id="rId41" xr:uid="{47F34AB3-0A0A-412F-8FE1-03EF5CACC9CA}"/>
+    <hyperlink ref="F60" r:id="rId42" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-complementar/2022/59/583/lei-complementar-n-583-2022-dispoe-sobre-aumento-salarial-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=aumento%20salarial" xr:uid="{9456DAAA-0A8A-485D-A402-82BED62E4A97}"/>
+    <hyperlink ref="F57" r:id="rId43" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2025/63/630/lei-ordinaria-n-630-2025-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{64BC75ED-1964-4204-BAFA-49F3A4083336}"/>
+    <hyperlink ref="F58" r:id="rId44" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2024/62/614/lei-ordinaria-n-614-2024-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{0661ED8C-7E04-4235-BDA6-165CAA2FD04B}"/>
+    <hyperlink ref="F59" r:id="rId45" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2023/59/588/lei-ordinaria-n-588-2023-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{4A341ABB-8BE7-4A6E-B4C1-532DBB4378D2}"/>
+    <hyperlink ref="F61" r:id="rId46" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2021/54/534/lei-ordinaria-n-534-2021-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{95B75048-0C9A-47CB-8A73-3D8052953EA1}"/>
+    <hyperlink ref="F62" r:id="rId47" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2020/52/516/lei-ordinaria-n-516-2020-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{46529EB6-AC15-4D01-B558-28DB00531128}"/>
+    <hyperlink ref="F64" r:id="rId48" xr:uid="{EE42FF6B-39FA-43BE-8F7C-A56762A03BE5}"/>
+    <hyperlink ref="F65" r:id="rId49" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2024/232/2320/lei-ordinaria-n-2320-2024-autoriza-revisao-geral-da-remuneracao-e-os-subsidios-dos-servidores-publicos-e-agentes-politicos-dos-poderes-executivo-e-legislativo-do-municipio-nos-termos-do-artigo-7-caput-iv-e-o-do-artigo-39-3-da-constituicao-federal-extensivo-aos-conselheiros-tutelares-e-aos-proventos-dos-inativos-e-pensionistas?q=Revis%C3%A3o+geraL" xr:uid="{4F7B275E-5955-4B1B-94E6-A35B6D80FEE2}"/>
+    <hyperlink ref="F69" r:id="rId50" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2021/218/2180/lei-ordinaria-n-2180-2021-suspende-os-efeitos-da-lei-municipal-n-2147-2021-que-autoriza-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-e-da-outras-providencias?q=Revis%E3o%20geraL" xr:uid="{EB57F7DB-CDEF-4A7C-9E25-23B1204FA785}"/>
+    <hyperlink ref="F70" r:id="rId51" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2020/211/2107/lei-ordinaria-n-2107-2020-autoriza-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-a-aplicacao-do-artigo-7-inciso-iv-e-art-39-3-da-constituicao-federal-a-remuneracao-dos-servidores-publicos-o-reajuste-dos-proventos-dos-inativos-e-pensionistas-a-recomposicao-dos-subsidios-dos-agentes-politicos-e-fixa-os-pisos-nacionais-minimos-para-os-integrantes-do-magisterio-municipal-11739-2008-e-da-outras-providencias?q=Revis%E3o%20geraL" xr:uid="{924B3E23-6A28-4DA7-BF55-853A35BD0084}"/>
+    <hyperlink ref="F67" r:id="rId52" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2021/220/2198/lei-ordinaria-n-2198-2021-autoriza-revisao-geral-da-remuneracao-dos-servidores-publicos-autoriza-a-aplicacao-do-artigo-7-caput-iv-e-o-do-artigo-39-3-da-constituicao-federal-a-remuneracao-dos-servidores-publicos-e-autoriza-o-reajuste-dos-proventos-dos-inativos-e-pensionistas?q=2.198" xr:uid="{D3688214-1F73-4C24-86E5-7E744B395889}"/>
+    <hyperlink ref="F68" r:id="rId53" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2021/220/2197/lei-ordinaria-n-2197-2021-autoriza-revisao-geral-da-remuneracao-dos-servidores-publicos-autoriza-a-aplicacao-do-artigo-7-caput-iv-e-o-do-artigo-39-3-da-constituicao-federal-a-remuneracao-dos-servidores-publicos-e-autoriza-o-reajuste-dos-proventos-dos-inativos-e-pensionistas?q=2.197" xr:uid="{824C9DCD-78D8-43FD-8DB5-0E165BC5D312}"/>
+    <hyperlink ref="F66" r:id="rId54" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2023/226/2251/lei-ordinaria-n-2251-2023-autoriza-revisao-geral-da-remuneracao-e-os-subsidios-dos-servidores-publicos-e-agentes-politicos-dos-poderes-executivo-e-legislativo-do-municipio-nos-termos-do-artigo-7-caput-iv-e-o-do-artigo-39-3-da-constituicao-federal-extensivo-aos-conselheiros-tutelares-e-aos-proventos-dos-inativos-e-pensionistas?q=Autoriza%20revis%E3o%20geral%20da%20remunera%E7%E3o" xr:uid="{7E99F84F-40DA-489D-BFB8-FC337539CA92}"/>
+    <hyperlink ref="F27" r:id="rId55" xr:uid="{6761F2DF-2A70-4664-8013-B14C436BF884}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId55"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId56"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
added dados de 2026
</commit_message>
<xml_diff>
--- a/data/dados.xlsx
+++ b/data/dados.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\reajuste\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D306AA63-91AF-4A34-A41E-000F1245219E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{955DB961-ADD9-4905-BB7A-D2F84A7F6B90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{BE2A1F3B-6535-41F1-9783-CEB15E5262F6}"/>
+    <workbookView xWindow="21480" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{BE2A1F3B-6535-41F1-9783-CEB15E5262F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
     <sheet name="Planilha2" sheetId="2" r:id="rId2"/>
+    <sheet name="Planilha3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="86">
   <si>
     <t>Cafeara</t>
   </si>
@@ -280,13 +281,28 @@
   </si>
   <si>
     <t>https://www.diariomunicipal.com.br/amp/materia/732EB9FD/f71481bba070e988d1c4ee95c9001e57f71481bba070e988d1c4ee95c9001e57</t>
+  </si>
+  <si>
+    <t>https://leismunicipais.com.br/a/pr/c/cafeara/lei-ordinaria/2026/70/698/lei-ordinaria-n-698-2026-autoriza-o-executivo-municipal-a-conceder-recomposicao-geral-anual-aos-servidores-publicos-municipais-e-aos-agentes-politicos-do-poder-executivo-municipal-de-cafeara-e-da-outras-providencias?q=698</t>
+  </si>
+  <si>
+    <t>https://leis.org/municipais/pr/santa-fe/lei/lei-ordinaria/2026/2453/lei-ordinaria-n-2453-2026-autoriza-revisao-geral-da-remuneracao-dos-servidores-publicos-dos-poderes-executivo-e-legislativo-do-municipio-nos-termos-do-artigo-7-caput-iv-e-do-artigo-39-3-da-constituicao-federal-extensivo-aos-proventos-dos-inativos-e-pensionistas</t>
+  </si>
+  <si>
+    <t>https://leis.org/municipais/pr/prado-ferreira/lei/lei-ordinaria/2026/658/lei-ordinaria-n-658-2026-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias</t>
+  </si>
+  <si>
+    <t>https://leis.org/municipais/pr/primeiro-de-maio/lei/lei-ordinaria/2026/1053/lei-ordinaria-n-1053-2026-dispoe-sobre-a-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-municipais-de-primeiro-de-maio-e-da-outras-providencias</t>
+  </si>
+  <si>
+    <t>https://www.diariomunicipal.com.br/amp/materia/770D27C0/8df711b55df2c192081af57b2fcc270b8df711b55df2c192081af57b2fcc270b</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -336,8 +352,21 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF222222"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -347,6 +376,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -360,11 +395,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -400,11 +436,22 @@
     <xf numFmtId="10" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="10" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentagem" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -736,7 +783,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95A9F774-A2B7-43E0-89BB-A01627A8B05C}">
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:G80"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.42578125" style="3" bestFit="1" customWidth="1"/>
@@ -889,7 +936,7 @@
       <c r="A10" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="20">
         <v>2026</v>
       </c>
       <c r="C10" s="7">
@@ -1032,15 +1079,17 @@
         <v>28</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="A19" s="4"/>
       <c r="C19" s="7"/>
+      <c r="G19" s="8"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B20" s="5">
-        <v>2025</v>
+      <c r="B20" s="20">
+        <v>2026</v>
       </c>
       <c r="C20" s="7">
         <v>0.1</v>
@@ -1052,7 +1101,7 @@
         <v>2648</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>17</v>
+        <v>81</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -1060,10 +1109,10 @@
         <v>0</v>
       </c>
       <c r="B21" s="5">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C21" s="7">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="D21" s="14">
         <v>4103404</v>
@@ -1072,7 +1121,7 @@
         <v>2648</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -1080,10 +1129,10 @@
         <v>0</v>
       </c>
       <c r="B22" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C22" s="7">
-        <v>0.2</v>
+        <v>0.05</v>
       </c>
       <c r="D22" s="14">
         <v>4103404</v>
@@ -1092,7 +1141,7 @@
         <v>2648</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
@@ -1100,10 +1149,10 @@
         <v>0</v>
       </c>
       <c r="B23" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C23" s="7">
-        <v>0.16059999999999999</v>
+        <v>0.2</v>
       </c>
       <c r="D23" s="14">
         <v>4103404</v>
@@ -1112,7 +1161,7 @@
         <v>2648</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -1120,10 +1169,10 @@
         <v>0</v>
       </c>
       <c r="B24" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C24" s="7">
-        <v>4.5199999999999997E-2</v>
+        <v>0.16059999999999999</v>
       </c>
       <c r="D24" s="14">
         <v>4103404</v>
@@ -1132,7 +1181,7 @@
         <v>2648</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
@@ -1140,10 +1189,10 @@
         <v>0</v>
       </c>
       <c r="B25" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C25" s="7">
-        <v>0.05</v>
+        <v>4.5199999999999997E-2</v>
       </c>
       <c r="D25" s="14">
         <v>4103404</v>
@@ -1152,43 +1201,43 @@
         <v>2648</v>
       </c>
       <c r="F25" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B26" s="5">
+        <v>2020</v>
+      </c>
+      <c r="C26" s="7">
+        <v>0.05</v>
+      </c>
+      <c r="D26" s="14">
+        <v>4103404</v>
+      </c>
+      <c r="E26" s="14">
+        <v>2648</v>
+      </c>
+      <c r="F26" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="C26" s="7"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-    </row>
-    <row r="27" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="B27" s="5">
-        <v>2026</v>
-      </c>
-      <c r="C27" s="7">
-        <v>4.2599999999999999E-2</v>
-      </c>
-      <c r="D27" s="14">
-        <v>4105102</v>
-      </c>
-      <c r="E27" s="14">
-        <v>10903</v>
-      </c>
-      <c r="F27" s="10" t="s">
-        <v>80</v>
-      </c>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="C27" s="7"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="5">
-        <v>2025</v>
+      <c r="B28" s="20">
+        <v>2026</v>
       </c>
       <c r="C28" s="7">
-        <v>0.05</v>
+        <v>4.2599999999999999E-2</v>
       </c>
       <c r="D28" s="14">
         <v>4105102</v>
@@ -1197,7 +1246,7 @@
         <v>10903</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>22</v>
+        <v>80</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
@@ -1205,7 +1254,7 @@
         <v>52</v>
       </c>
       <c r="B29" s="5">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C29" s="7">
         <v>0.05</v>
@@ -1217,7 +1266,7 @@
         <v>10903</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
@@ -1225,10 +1274,10 @@
         <v>52</v>
       </c>
       <c r="B30" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C30" s="7">
-        <v>5.9299999999999999E-2</v>
+        <v>0.05</v>
       </c>
       <c r="D30" s="14">
         <v>4105102</v>
@@ -1237,7 +1286,7 @@
         <v>10903</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -1245,10 +1294,10 @@
         <v>52</v>
       </c>
       <c r="B31" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C31" s="7">
-        <v>0.1016</v>
+        <v>5.9299999999999999E-2</v>
       </c>
       <c r="D31" s="14">
         <v>4105102</v>
@@ -1257,7 +1306,7 @@
         <v>10903</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
@@ -1265,10 +1314,10 @@
         <v>52</v>
       </c>
       <c r="B32" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C32" s="7">
-        <v>4.5199999999999997E-2</v>
+        <v>0.1016</v>
       </c>
       <c r="D32" s="14">
         <v>4105102</v>
@@ -1277,7 +1326,7 @@
         <v>10903</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
@@ -1285,10 +1334,10 @@
         <v>52</v>
       </c>
       <c r="B33" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C33" s="7">
-        <v>4.48E-2</v>
+        <v>4.5199999999999997E-2</v>
       </c>
       <c r="D33" s="14">
         <v>4105102</v>
@@ -1297,43 +1346,43 @@
         <v>10903</v>
       </c>
       <c r="F33" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A34" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B34" s="5">
+        <v>2020</v>
+      </c>
+      <c r="C34" s="7">
+        <v>4.48E-2</v>
+      </c>
+      <c r="D34" s="14">
+        <v>4105102</v>
+      </c>
+      <c r="E34" s="14">
+        <v>10903</v>
+      </c>
+      <c r="F34" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C34" s="7"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-    </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A35" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B35" s="5">
-        <v>2025</v>
-      </c>
-      <c r="C35" s="7">
-        <v>0.05</v>
-      </c>
-      <c r="D35" s="14">
-        <v>4113809</v>
-      </c>
-      <c r="E35" s="14">
-        <v>4929</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>30</v>
-      </c>
+      <c r="C35" s="7"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="14"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
         <v>51</v>
       </c>
       <c r="B36" s="5">
-        <v>2024</v>
-      </c>
-      <c r="C36" s="7">
-        <v>0.05</v>
+        <v>2026</v>
+      </c>
+      <c r="C36" s="21">
+        <v>3.9E-2</v>
       </c>
       <c r="D36" s="14">
         <v>4113809</v>
@@ -1342,7 +1391,7 @@
         <v>4929</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>31</v>
+        <v>85</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
@@ -1350,10 +1399,10 @@
         <v>51</v>
       </c>
       <c r="B37" s="5">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="C37" s="7">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
       <c r="D37" s="14">
         <v>4113809</v>
@@ -1362,7 +1411,7 @@
         <v>4929</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
@@ -1370,10 +1419,10 @@
         <v>51</v>
       </c>
       <c r="B38" s="5">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C38" s="7">
-        <v>5.45E-2</v>
+        <v>0.05</v>
       </c>
       <c r="D38" s="14">
         <v>4113809</v>
@@ -1382,7 +1431,7 @@
         <v>4929</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
@@ -1390,10 +1439,10 @@
         <v>51</v>
       </c>
       <c r="B39" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C39" s="7">
-        <v>0.1016</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="D39" s="14">
         <v>4113809</v>
@@ -1402,7 +1451,7 @@
         <v>4929</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
@@ -1410,14 +1459,19 @@
         <v>51</v>
       </c>
       <c r="B40" s="5">
-        <v>2021</v>
-      </c>
-      <c r="C40" s="7"/>
+        <v>2022</v>
+      </c>
+      <c r="C40" s="7">
+        <v>5.45E-2</v>
+      </c>
       <c r="D40" s="14">
         <v>4113809</v>
       </c>
       <c r="E40" s="14">
         <v>4929</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
@@ -1425,10 +1479,10 @@
         <v>51</v>
       </c>
       <c r="B41" s="5">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="C41" s="7">
-        <v>4.48E-2</v>
+        <v>0.1016</v>
       </c>
       <c r="D41" s="14">
         <v>4113809</v>
@@ -1437,72 +1491,62 @@
         <v>4929</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C42" s="7"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
+      <c r="A42" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B42" s="5">
+        <v>2021</v>
+      </c>
+      <c r="C42" s="19"/>
+      <c r="D42" s="14">
+        <v>4113809</v>
+      </c>
+      <c r="E42" s="14">
+        <v>4929</v>
+      </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B43" s="5">
-        <v>2025</v>
+        <v>2020</v>
       </c>
       <c r="C43" s="7">
-        <v>0.05</v>
+        <v>4.48E-2</v>
       </c>
       <c r="D43" s="14">
-        <v>4111902</v>
+        <v>4113809</v>
       </c>
       <c r="E43" s="14">
-        <v>15908</v>
+        <v>4929</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A44" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B44" s="5">
-        <v>2024</v>
-      </c>
-      <c r="C44" s="7">
-        <v>0.05</v>
-      </c>
-      <c r="D44" s="14">
-        <v>4111902</v>
-      </c>
-      <c r="E44" s="14">
-        <v>15908</v>
-      </c>
-      <c r="F44" s="3" t="s">
-        <v>36</v>
-      </c>
+      <c r="C44" s="7"/>
+      <c r="D44" s="14"/>
+      <c r="E44" s="14"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="3" t="s">
         <v>50</v>
       </c>
       <c r="B45" s="5">
-        <v>2023</v>
-      </c>
-      <c r="C45" s="7">
-        <v>0.14949999999999999</v>
-      </c>
+        <v>2026</v>
+      </c>
+      <c r="C45" s="19"/>
       <c r="D45" s="14">
         <v>4111902</v>
       </c>
       <c r="E45" s="14">
         <v>15908</v>
-      </c>
-      <c r="F45" s="3" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
@@ -1510,10 +1554,10 @@
         <v>50</v>
       </c>
       <c r="B46" s="5">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="C46" s="7">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="D46" s="14">
         <v>4111902</v>
@@ -1522,7 +1566,7 @@
         <v>15908</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
@@ -1530,10 +1574,10 @@
         <v>50</v>
       </c>
       <c r="B47" s="5">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C47" s="7">
-        <v>5.5300000000000002E-2</v>
+        <v>0.05</v>
       </c>
       <c r="D47" s="14">
         <v>4111902</v>
@@ -1542,7 +1586,7 @@
         <v>15908</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
@@ -1550,10 +1594,10 @@
         <v>50</v>
       </c>
       <c r="B48" s="5">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="C48" s="7">
-        <v>2.2499999999999999E-2</v>
+        <v>0.14949999999999999</v>
       </c>
       <c r="D48" s="14">
         <v>4111902</v>
@@ -1562,83 +1606,83 @@
         <v>15908</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C49" s="7"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="14"/>
+      <c r="A49" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B49" s="5">
+        <v>2022</v>
+      </c>
+      <c r="C49" s="7">
+        <v>0.15</v>
+      </c>
+      <c r="D49" s="14">
+        <v>4111902</v>
+      </c>
+      <c r="E49" s="14">
+        <v>15908</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="B50" s="5">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="C50" s="7">
-        <v>4.8300000000000003E-2</v>
+        <v>5.5300000000000002E-2</v>
       </c>
       <c r="D50" s="14">
-        <v>4120507</v>
+        <v>4111902</v>
       </c>
       <c r="E50" s="14">
-        <v>10064</v>
+        <v>15908</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="B51" s="5">
-        <v>2024</v>
+        <v>2020</v>
       </c>
       <c r="C51" s="7">
-        <v>0.11460000000000001</v>
+        <v>2.2499999999999999E-2</v>
       </c>
       <c r="D51" s="14">
-        <v>4120507</v>
+        <v>4111902</v>
       </c>
       <c r="E51" s="14">
-        <v>10064</v>
+        <v>15908</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A52" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B52" s="5">
-        <v>2023</v>
-      </c>
-      <c r="C52" s="7">
-        <v>0.1263</v>
-      </c>
-      <c r="D52" s="14">
-        <v>4120507</v>
-      </c>
-      <c r="E52" s="14">
-        <v>10064</v>
-      </c>
-      <c r="F52" s="3" t="s">
-        <v>44</v>
-      </c>
+      <c r="C52" s="7"/>
+      <c r="D52" s="14"/>
+      <c r="E52" s="14"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
         <v>43</v>
       </c>
       <c r="B53" s="5">
-        <v>2022</v>
-      </c>
-      <c r="C53" s="7">
-        <v>0.15</v>
+        <v>2026</v>
+      </c>
+      <c r="C53" s="21">
+        <v>4.2599999999999999E-2</v>
       </c>
       <c r="D53" s="14">
         <v>4120507</v>
@@ -1647,7 +1691,7 @@
         <v>10064</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>48</v>
+        <v>84</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
@@ -1655,10 +1699,10 @@
         <v>43</v>
       </c>
       <c r="B54" s="5">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="C54" s="7">
-        <v>4.5199999999999997E-2</v>
+        <v>4.8300000000000003E-2</v>
       </c>
       <c r="D54" s="14">
         <v>4120507</v>
@@ -1667,7 +1711,7 @@
         <v>10064</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
@@ -1675,10 +1719,10 @@
         <v>43</v>
       </c>
       <c r="B55" s="5">
-        <v>2020</v>
+        <v>2024</v>
       </c>
       <c r="C55" s="7">
-        <v>7.3178999999999994E-2</v>
+        <v>0.11460000000000001</v>
       </c>
       <c r="D55" s="14">
         <v>4120507</v>
@@ -1687,102 +1731,103 @@
         <v>10064</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D56" s="14"/>
-      <c r="E56" s="14"/>
+      <c r="A56" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B56" s="5">
+        <v>2023</v>
+      </c>
+      <c r="C56" s="7">
+        <v>0.1263</v>
+      </c>
+      <c r="D56" s="14">
+        <v>4120507</v>
+      </c>
+      <c r="E56" s="14">
+        <v>10064</v>
+      </c>
+      <c r="F56" s="3" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="B57" s="5">
-        <v>2025</v>
-      </c>
-      <c r="C57" s="17">
-        <v>4.8300000000000003E-2</v>
+        <v>2022</v>
+      </c>
+      <c r="C57" s="7">
+        <v>0.15</v>
       </c>
       <c r="D57" s="14">
-        <v>4120333</v>
+        <v>4120507</v>
       </c>
       <c r="E57" s="14">
-        <v>3816</v>
+        <v>10064</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" s="3" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="B58" s="5">
-        <v>2024</v>
-      </c>
-      <c r="C58" s="17">
-        <v>4.6199999999999998E-2</v>
+        <v>2021</v>
+      </c>
+      <c r="C58" s="7">
+        <v>4.5199999999999997E-2</v>
       </c>
       <c r="D58" s="14">
-        <v>4120333</v>
+        <v>4120507</v>
       </c>
       <c r="E58" s="14">
-        <v>3816</v>
+        <v>10064</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="B59" s="5">
-        <v>2023</v>
-      </c>
-      <c r="C59" s="17">
-        <v>5.9299999999999999E-2</v>
+        <v>2020</v>
+      </c>
+      <c r="C59" s="7">
+        <v>7.3178999999999994E-2</v>
       </c>
       <c r="D59" s="14">
-        <v>4120333</v>
+        <v>4120507</v>
       </c>
       <c r="E59" s="14">
-        <v>3816</v>
+        <v>10064</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A60" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B60" s="5">
-        <v>2022</v>
-      </c>
-      <c r="C60" s="17">
-        <v>0.1</v>
-      </c>
-      <c r="D60" s="14">
-        <v>4120333</v>
-      </c>
-      <c r="E60" s="14">
-        <v>3816</v>
-      </c>
-      <c r="F60" s="3" t="s">
-        <v>55</v>
-      </c>
+      <c r="C60" s="7"/>
+      <c r="D60" s="14"/>
+      <c r="E60" s="14"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
         <v>54</v>
       </c>
       <c r="B61" s="5">
-        <v>2021</v>
-      </c>
-      <c r="C61" s="17">
-        <v>4.5199999999999997E-2</v>
+        <v>2026</v>
+      </c>
+      <c r="C61" s="7">
+        <v>4.4400000000000002E-2</v>
       </c>
       <c r="D61" s="14">
         <v>4120333</v>
@@ -1791,7 +1836,7 @@
         <v>3816</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>59</v>
+        <v>83</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.2">
@@ -1799,10 +1844,10 @@
         <v>54</v>
       </c>
       <c r="B62" s="5">
-        <v>2020</v>
-      </c>
-      <c r="C62" s="17">
-        <v>4.3099999999999999E-2</v>
+        <v>2025</v>
+      </c>
+      <c r="C62" s="7">
+        <v>4.8300000000000003E-2</v>
       </c>
       <c r="D62" s="14">
         <v>4120333</v>
@@ -1811,121 +1856,123 @@
         <v>3816</v>
       </c>
       <c r="F62" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A63" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B63" s="5">
+        <v>2024</v>
+      </c>
+      <c r="C63" s="7">
+        <v>4.6199999999999998E-2</v>
+      </c>
+      <c r="D63" s="14">
+        <v>4120333</v>
+      </c>
+      <c r="E63" s="14">
+        <v>3816</v>
+      </c>
+      <c r="F63" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A64" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B64" s="5">
+        <v>2023</v>
+      </c>
+      <c r="C64" s="7">
+        <v>5.9299999999999999E-2</v>
+      </c>
+      <c r="D64" s="14">
+        <v>4120333</v>
+      </c>
+      <c r="E64" s="14">
+        <v>3816</v>
+      </c>
+      <c r="F64" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A65" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B65" s="5">
+        <v>2022</v>
+      </c>
+      <c r="C65" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="D65" s="14">
+        <v>4120333</v>
+      </c>
+      <c r="E65" s="14">
+        <v>3816</v>
+      </c>
+      <c r="F65" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A66" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B66" s="5">
+        <v>2021</v>
+      </c>
+      <c r="C66" s="7">
+        <v>4.5199999999999997E-2</v>
+      </c>
+      <c r="D66" s="14">
+        <v>4120333</v>
+      </c>
+      <c r="E66" s="14">
+        <v>3816</v>
+      </c>
+      <c r="F66" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A67" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B67" s="5">
+        <v>2020</v>
+      </c>
+      <c r="C67" s="7">
+        <v>4.3099999999999999E-2</v>
+      </c>
+      <c r="D67" s="14">
+        <v>4120333</v>
+      </c>
+      <c r="E67" s="14">
+        <v>3816</v>
+      </c>
+      <c r="F67" s="3" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E63" s="14"/>
-    </row>
-    <row r="64" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A64" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B64" s="5">
-        <v>2025</v>
-      </c>
-      <c r="C64" s="7">
-        <v>0.05</v>
-      </c>
-      <c r="D64" s="14">
-        <v>4123402</v>
-      </c>
-      <c r="E64" s="14">
-        <v>11730</v>
-      </c>
-      <c r="F64" s="10" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A65" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B65" s="5">
-        <v>2024</v>
-      </c>
-      <c r="C65" s="7">
-        <v>0.04</v>
-      </c>
-      <c r="D65" s="14">
-        <v>4123402</v>
-      </c>
-      <c r="E65" s="14">
-        <v>11730</v>
-      </c>
-      <c r="F65" s="10" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A66" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B66" s="5">
-        <v>2023</v>
-      </c>
-      <c r="C66" s="7">
-        <v>0.1</v>
-      </c>
-      <c r="D66" s="14">
-        <v>4123402</v>
-      </c>
-      <c r="E66" s="14">
-        <v>11730</v>
-      </c>
-      <c r="F66" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A67" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B67" s="5">
-        <v>2022</v>
-      </c>
-      <c r="C67" s="7">
-        <v>0.15</v>
-      </c>
-      <c r="D67" s="14">
-        <v>4123402</v>
-      </c>
-      <c r="E67" s="14">
-        <v>11730</v>
-      </c>
-      <c r="F67" s="10" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A68" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B68" s="5">
-        <v>2022</v>
-      </c>
-      <c r="C68" s="7">
-        <v>0.15</v>
-      </c>
-      <c r="D68" s="14">
-        <v>4123402</v>
-      </c>
-      <c r="E68" s="14">
-        <v>11730</v>
-      </c>
-      <c r="F68" s="10" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="C68" s="7"/>
+      <c r="D68" s="14"/>
+      <c r="E68" s="14"/>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" s="3" t="s">
         <v>70</v>
       </c>
       <c r="B69" s="5">
-        <v>2021</v>
+        <v>2026</v>
       </c>
       <c r="C69" s="7">
-        <v>4.5199999999999997E-2</v>
+        <v>0.04</v>
       </c>
       <c r="D69" s="14">
         <v>4123402</v>
@@ -1933,8 +1980,8 @@
       <c r="E69" s="14">
         <v>11730</v>
       </c>
-      <c r="F69" s="10" t="s">
-        <v>73</v>
+      <c r="F69" s="3" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="70" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
@@ -1942,10 +1989,10 @@
         <v>70</v>
       </c>
       <c r="B70" s="5">
-        <v>2020</v>
+        <v>2025</v>
       </c>
       <c r="C70" s="7">
-        <v>4.3099999999999999E-2</v>
+        <v>0.05</v>
       </c>
       <c r="D70" s="14">
         <v>4123402</v>
@@ -1953,21 +2000,141 @@
       <c r="E70" s="14">
         <v>11730</v>
       </c>
-      <c r="F70" s="10" t="s">
+      <c r="F70" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="A71" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B71" s="5">
+        <v>2024</v>
+      </c>
+      <c r="C71" s="7">
+        <v>0.04</v>
+      </c>
+      <c r="D71" s="14">
+        <v>4123402</v>
+      </c>
+      <c r="E71" s="14">
+        <v>11730</v>
+      </c>
+      <c r="F71" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="A72" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B72" s="5">
+        <v>2023</v>
+      </c>
+      <c r="C72" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="D72" s="14">
+        <v>4123402</v>
+      </c>
+      <c r="E72" s="14">
+        <v>11730</v>
+      </c>
+      <c r="F72" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="A73" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B73" s="5">
+        <v>2022</v>
+      </c>
+      <c r="C73" s="7">
+        <v>0.15</v>
+      </c>
+      <c r="D73" s="14">
+        <v>4123402</v>
+      </c>
+      <c r="E73" s="14">
+        <v>11730</v>
+      </c>
+      <c r="F73" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="A74" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B74" s="5">
+        <v>2022</v>
+      </c>
+      <c r="C74" s="7">
+        <v>0.15</v>
+      </c>
+      <c r="D74" s="14">
+        <v>4123402</v>
+      </c>
+      <c r="E74" s="14">
+        <v>11730</v>
+      </c>
+      <c r="F74" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="A75" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B75" s="5">
+        <v>2021</v>
+      </c>
+      <c r="C75" s="7">
+        <v>4.5199999999999997E-2</v>
+      </c>
+      <c r="D75" s="14">
+        <v>4123402</v>
+      </c>
+      <c r="E75" s="14">
+        <v>11730</v>
+      </c>
+      <c r="F75" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="A76" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B76" s="5">
+        <v>2020</v>
+      </c>
+      <c r="C76" s="7">
+        <v>4.3099999999999999E-2</v>
+      </c>
+      <c r="D76" s="14">
+        <v>4123402</v>
+      </c>
+      <c r="E76" s="14">
+        <v>11730</v>
+      </c>
+      <c r="F76" s="3" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E71" s="14"/>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E72" s="14"/>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E73" s="14"/>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E74" s="14"/>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E77" s="14"/>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E78" s="14"/>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E79" s="14"/>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E80" s="14"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1979,56 +2146,61 @@
     <hyperlink ref="G5" r:id="rId6" xr:uid="{DF98840A-BED1-49E1-B92D-46CC476DBA26}"/>
     <hyperlink ref="G6" r:id="rId7" xr:uid="{2035362C-9A91-4B81-829D-3D0C4FA771DF}"/>
     <hyperlink ref="G14" r:id="rId8" xr:uid="{CE999FD0-8CBC-4BEA-84BE-95B4E1C3A1C5}"/>
-    <hyperlink ref="F22" r:id="rId9" display="https://leis.org/municipais/pr/cafeara/lei/lei-ordinaria/2023/609/lei-ordinaria-n-609-2023-autoriza-o-executivo-municipal-a-conceder-recomposicao-geral-anual-aos-servidores-publicos-municipais-e-agentes-politicos-do-poder-executivo-municipal-de-cafeara-e-da-outras-providencias" xr:uid="{C3275B82-C56D-4C85-BA27-2F2BD690BB16}"/>
-    <hyperlink ref="F20" r:id="rId10" display="https://leis.org/municipais/pr/cafeara/lei/lei-complementar/2025/669/lei-complementar-n-669-2025-autoriza-o-executivo-municipal-a-conceder-recomposicao-geral-anual-aos-servidores-publicos-municipais-e-agentes-politicos-do-poder-executivo-municipal-de-cafeara-e-da-outras-providencias?termo=RECOMPOSI%C3%87%C3%83O%20GERAL%20ANUAL" xr:uid="{A7EAD4F8-68E0-41D4-AE50-5A0B782E8B8F}"/>
-    <hyperlink ref="F21" r:id="rId11" display="https://leis.org/municipais/pr/cafeara/lei/lei-ordinaria/2024/636/lei-ordinaria-n-636-2024-autoriza-o-executivo-municipal-a-conceder-recomposicao-geral-anual-aos-servidores-publicos-municipais-e-agentes-politicos-do-poder-executivo-municipal-de-cafeara-e-da-outras-providencias?termo=RECOMPOSI%C3%87%C3%83O%20GERAL%20ANUAL" xr:uid="{23D66F80-65EE-4A0F-8144-F36DB20450EF}"/>
-    <hyperlink ref="F23" r:id="rId12" display="https://leis.org/municipais/pr/cafeara/lei/lei-ordinaria/2022/587/lei-ordinaria-n-587-2022-autoriza-o-executivo-municipal-a-conceder-recomposicao-geral-anual-aos-servidores-publicos-municipais-e-agentes-politicos-do-poder-executivo-municipal-de-cafeara-e-da-outras-providencias?termo=RECOMPOSI%C3%87%C3%83O%20GERAL%20ANUAL" xr:uid="{1B38F967-CA98-456B-9E39-53D8B29C2593}"/>
-    <hyperlink ref="F24" r:id="rId13" display="https://leis.org/municipais/pr/cafeara/lei/lei-ordinaria/2021/563/lei-ordinaria-n-563-2021-autoriza-o-executivo-municipal-a-conceder-recomposicao-geral-anual-aos-servidores-publicos-municipais-e-agentes-politicos-do-poder-executivo-municipal-de-cafeara-e-da-outras-providencias?termo=RECOMPOSI%C3%87%C3%83O%20GERAL%20ANUAL" xr:uid="{2F2E9EFC-04E5-4D6C-ADAE-3D1C1FE4D8C2}"/>
-    <hyperlink ref="F25" r:id="rId14" display="https://leis.org/municipais/pr/cafeara/lei/lei-ordinaria/2020/542/lei-ordinaria-n-542-2020-autoriza-o-executivo-municipal-a-conceder-recomposicao-geral-anual-aos-servidores-publicos-municipais-e-agentes-politicos-do-poder-executivo-municipal-de-cafeara-e-revisao-salarial-aos-servidores-publicos-municipais-e-da-outras-providencias?termo=RECOMPOSI%C3%87%C3%83O%20GERAL%20ANUAL" xr:uid="{CE150FB9-81B7-4D95-A8CF-6EF4FEC69817}"/>
-    <hyperlink ref="F28" r:id="rId15" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2025/325/3248/lei-ordinaria-n-3248-2025-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-com-excecao-dos-subsidios-dos-agentes-politicos?q=reajuste" xr:uid="{14532045-718C-41E1-8B54-50EFD37FBDB7}"/>
-    <hyperlink ref="F29" r:id="rId16" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2024/322/3211/lei-ordinaria-n-3211-2024-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-inclusive-sobre-os-subsidios-dos-agentes-politicos?q=reajuste" xr:uid="{38AE6B04-78B2-4EB9-9571-DB2D521C73B5}"/>
-    <hyperlink ref="F30" r:id="rId17" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2023/317/3170/lei-ordinaria-n-3170-2023-autoriza-a-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-inclusive-sobre-os-subsidios-dos-agentes-politicos?q=reajuste" xr:uid="{4CF69429-E3A8-42D6-85E9-C1B4DF636DEA}"/>
-    <hyperlink ref="F31" r:id="rId18" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2022/314/3132/lei-ordinaria-n-3132-2022-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-inclusive-sobre-os-subsidios-dos-agentes-politicos?q=reajuste" xr:uid="{55BFE9D4-B84C-4424-B8D7-86FC64A9AB3E}"/>
-    <hyperlink ref="F32" r:id="rId19" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2021/310/3097/lei-ordinaria-n-3097-2021-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao?q=reajuste" xr:uid="{87876156-98C2-4000-91CE-7C8AD0B3476E}"/>
-    <hyperlink ref="F33" r:id="rId20" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2020/305/3045/lei-ordinaria-n-3045-2020-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-inclusive-sobre-os-subsidios-dos-agentes-politicos-bem-como-adequa-o-salario-dos-servidores-do-quadro-do-magisterio-publico-municipal-ao-piso-salarial-profissional-nacional?q=reajuste" xr:uid="{DF65B76A-65AA-4C35-A537-F477C0AB6BF4}"/>
+    <hyperlink ref="F23" r:id="rId9" display="https://leis.org/municipais/pr/cafeara/lei/lei-ordinaria/2023/609/lei-ordinaria-n-609-2023-autoriza-o-executivo-municipal-a-conceder-recomposicao-geral-anual-aos-servidores-publicos-municipais-e-agentes-politicos-do-poder-executivo-municipal-de-cafeara-e-da-outras-providencias" xr:uid="{C3275B82-C56D-4C85-BA27-2F2BD690BB16}"/>
+    <hyperlink ref="F21" r:id="rId10" display="https://leis.org/municipais/pr/cafeara/lei/lei-complementar/2025/669/lei-complementar-n-669-2025-autoriza-o-executivo-municipal-a-conceder-recomposicao-geral-anual-aos-servidores-publicos-municipais-e-agentes-politicos-do-poder-executivo-municipal-de-cafeara-e-da-outras-providencias?termo=RECOMPOSI%C3%87%C3%83O%20GERAL%20ANUAL" xr:uid="{A7EAD4F8-68E0-41D4-AE50-5A0B782E8B8F}"/>
+    <hyperlink ref="F22" r:id="rId11" display="https://leis.org/municipais/pr/cafeara/lei/lei-ordinaria/2024/636/lei-ordinaria-n-636-2024-autoriza-o-executivo-municipal-a-conceder-recomposicao-geral-anual-aos-servidores-publicos-municipais-e-agentes-politicos-do-poder-executivo-municipal-de-cafeara-e-da-outras-providencias?termo=RECOMPOSI%C3%87%C3%83O%20GERAL%20ANUAL" xr:uid="{23D66F80-65EE-4A0F-8144-F36DB20450EF}"/>
+    <hyperlink ref="F24" r:id="rId12" display="https://leis.org/municipais/pr/cafeara/lei/lei-ordinaria/2022/587/lei-ordinaria-n-587-2022-autoriza-o-executivo-municipal-a-conceder-recomposicao-geral-anual-aos-servidores-publicos-municipais-e-agentes-politicos-do-poder-executivo-municipal-de-cafeara-e-da-outras-providencias?termo=RECOMPOSI%C3%87%C3%83O%20GERAL%20ANUAL" xr:uid="{1B38F967-CA98-456B-9E39-53D8B29C2593}"/>
+    <hyperlink ref="F25" r:id="rId13" display="https://leis.org/municipais/pr/cafeara/lei/lei-ordinaria/2021/563/lei-ordinaria-n-563-2021-autoriza-o-executivo-municipal-a-conceder-recomposicao-geral-anual-aos-servidores-publicos-municipais-e-agentes-politicos-do-poder-executivo-municipal-de-cafeara-e-da-outras-providencias?termo=RECOMPOSI%C3%87%C3%83O%20GERAL%20ANUAL" xr:uid="{2F2E9EFC-04E5-4D6C-ADAE-3D1C1FE4D8C2}"/>
+    <hyperlink ref="F26" r:id="rId14" display="https://leis.org/municipais/pr/cafeara/lei/lei-ordinaria/2020/542/lei-ordinaria-n-542-2020-autoriza-o-executivo-municipal-a-conceder-recomposicao-geral-anual-aos-servidores-publicos-municipais-e-agentes-politicos-do-poder-executivo-municipal-de-cafeara-e-revisao-salarial-aos-servidores-publicos-municipais-e-da-outras-providencias?termo=RECOMPOSI%C3%87%C3%83O%20GERAL%20ANUAL" xr:uid="{CE150FB9-81B7-4D95-A8CF-6EF4FEC69817}"/>
+    <hyperlink ref="F29" r:id="rId15" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2025/325/3248/lei-ordinaria-n-3248-2025-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-com-excecao-dos-subsidios-dos-agentes-politicos?q=reajuste" xr:uid="{14532045-718C-41E1-8B54-50EFD37FBDB7}"/>
+    <hyperlink ref="F30" r:id="rId16" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2024/322/3211/lei-ordinaria-n-3211-2024-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-inclusive-sobre-os-subsidios-dos-agentes-politicos?q=reajuste" xr:uid="{38AE6B04-78B2-4EB9-9571-DB2D521C73B5}"/>
+    <hyperlink ref="F31" r:id="rId17" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2023/317/3170/lei-ordinaria-n-3170-2023-autoriza-a-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-inclusive-sobre-os-subsidios-dos-agentes-politicos?q=reajuste" xr:uid="{4CF69429-E3A8-42D6-85E9-C1B4DF636DEA}"/>
+    <hyperlink ref="F32" r:id="rId18" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2022/314/3132/lei-ordinaria-n-3132-2022-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-inclusive-sobre-os-subsidios-dos-agentes-politicos?q=reajuste" xr:uid="{55BFE9D4-B84C-4424-B8D7-86FC64A9AB3E}"/>
+    <hyperlink ref="F33" r:id="rId19" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2021/310/3097/lei-ordinaria-n-3097-2021-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao?q=reajuste" xr:uid="{87876156-98C2-4000-91CE-7C8AD0B3476E}"/>
+    <hyperlink ref="F34" r:id="rId20" display="https://leismunicipais.com.br/a1/pr/c/centenario-do-sul/lei-ordinaria/2020/305/3045/lei-ordinaria-n-3045-2020-autoriza-o-chefe-do-poder-executivo-municipal-a-conceder-reposicao-salarial-nos-vencimentos-e-proventos-dos-servidores-ativos-inativos-e-pensionistas-efetivo-ou-em-comissao-inclusive-sobre-os-subsidios-dos-agentes-politicos-bem-como-adequa-o-salario-dos-servidores-do-quadro-do-magisterio-publico-municipal-ao-piso-salarial-profissional-nacional?q=reajuste" xr:uid="{DF65B76A-65AA-4C35-A537-F477C0AB6BF4}"/>
     <hyperlink ref="G18" r:id="rId21" xr:uid="{EC4616F6-7680-425A-9B5B-FA1377623831}"/>
     <hyperlink ref="F10" r:id="rId22" xr:uid="{5B0B0D6A-84BF-4334-B8E3-04EFE33A5016}"/>
     <hyperlink ref="F2" r:id="rId23" xr:uid="{5300EFF3-C77D-4044-9FEE-10FEE221CCA5}"/>
-    <hyperlink ref="F35" r:id="rId24" xr:uid="{0198FF07-6ABC-4FE0-BC94-9626A092EF1E}"/>
-    <hyperlink ref="F36" r:id="rId25" xr:uid="{9B9DADFC-147D-439F-A89B-8D7EC2EFFA45}"/>
-    <hyperlink ref="F37" r:id="rId26" xr:uid="{7B4312A5-B4D6-48C3-9967-D4A547A0F189}"/>
-    <hyperlink ref="F41" r:id="rId27" xr:uid="{B555F1DF-7AE0-4CE3-A746-A72DB71A3814}"/>
-    <hyperlink ref="F43" r:id="rId28" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2025/1/3/lei-ordinaria-n-3-2025-concede-recomposicao-e-reajuste-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{79AF655C-919A-4B59-8D63-6E9B71A0DFD8}"/>
-    <hyperlink ref="F44" r:id="rId29" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2024/1/6/lei-ordinaria-n-6-2024-concede-recomposicao-e-reajuste-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-e-recomposicao-inflacionaria-aos-agentes-politicos-do-poder-executivo-prefeito-vice-prefeito-e-secretarios-municipais-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{28DF2AEC-02FD-4904-92E4-8F1A46B7C53A}"/>
-    <hyperlink ref="F45" r:id="rId30" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2023/1/3/lei-ordinaria-n-3-2023-concede-recomposicao-e-reajuste-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-e-recomposicao-inflacionaria-aos-agentes-politicos-do-poder-executivo-prefeito-vice-prefeito-e-secretarios-municipais-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{D52BDBF7-13A5-4A80-A127-116B587657FB}"/>
-    <hyperlink ref="F46" r:id="rId31" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2022/1/5/lei-ordinaria-n-5-2022-concede-recomposicao-e-reajuste-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{3E75ABFE-1194-4B2F-AF68-D20DEC412ED8}"/>
-    <hyperlink ref="F47" r:id="rId32" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2021/1/5/lei-ordinaria-n-5-2021-concede-recomposicao-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{4FC8FEEE-0401-4369-8921-ED4B51F5562D}"/>
-    <hyperlink ref="F48" r:id="rId33" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2020/2/11/lei-ordinaria-n-11-2020-concede-recomposicao-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-e-ao-prefeito-vice-prefeito-e-secretarios-municipais-desta-municipalidade-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{4D8E764E-22B9-4B1F-A195-598C7E088B03}"/>
-    <hyperlink ref="F52" r:id="rId34" xr:uid="{469628B4-8B6D-46C9-A62E-832B5D06C62E}"/>
-    <hyperlink ref="F55" r:id="rId35" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2020/74/739/lei-ordinaria-n-739-2020-dispoe-sobre-a-revisao-geral-anual-do-subsidio-do-prefeito-vice-prefeito-vereadores-secretarios-as-municipais-e-remuneracao-do-s-servidor-es-comissionados-e-estatutario-do-poder-legislativo-do-municipio-de-primeiro-de-maio-e-da-outras-providencias?q=salarial%20" xr:uid="{8F367E47-ABB7-4AAB-A611-4BB40BDA61A3}"/>
-    <hyperlink ref="F50" r:id="rId36" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2025/97/970/lei-ordinaria-n-970-2025-dispoe-sobre-a-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-municipais-de-primeiro-de-maio-e-da-outras-providencias?q=revis%E3o%20geral%20anual%20" xr:uid="{9C1E9D0B-D3E4-4ECB-928C-3AB9384788C0}"/>
-    <hyperlink ref="F51" r:id="rId37" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2024/94/934/lei-ordinaria-n-934-2024-dispoe-sobre-a-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-municipais-de-primeiro-de-maio-e-da-outras-providencias?q=revis%E3o%20geral%20anual%20" xr:uid="{AF964D4D-7701-48C8-898F-A6225D73AC79}"/>
-    <hyperlink ref="F53" r:id="rId38" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2022/80/800/lei-ordinaria-n-800-2022-dispoe-sobre-a-revisao-geral-anual-do-subsidio-do-prefeito-vice-prefeito-vereadores-secretarios-as-municipais-e-remuneracao-do-s-servidor-es-comissionados-e-estatutario-do-poder-legislativo-do-municipio-de-primeiro-de-maio-e-da-outras-providencias?q=revis%E3o%20geral%20anual%20" xr:uid="{98F545B3-8D3D-44B1-AB35-4AC2759963EB}"/>
-    <hyperlink ref="F54" r:id="rId39" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2021/77/770/lei-ordinaria-n-770-2021-dispoe-sobre-a-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-municipais-de-primeiro-de-maio-e-da-outras-providencias?q=revis%E3o%20geral%20anual%20" xr:uid="{C52DDB23-FB88-489B-BD74-E79A0801ADF5}"/>
-    <hyperlink ref="F39" r:id="rId40" xr:uid="{878A7E66-55B4-4DAF-8A75-A1CF624BBEC7}"/>
-    <hyperlink ref="F38" r:id="rId41" xr:uid="{47F34AB3-0A0A-412F-8FE1-03EF5CACC9CA}"/>
-    <hyperlink ref="F60" r:id="rId42" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-complementar/2022/59/583/lei-complementar-n-583-2022-dispoe-sobre-aumento-salarial-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=aumento%20salarial" xr:uid="{9456DAAA-0A8A-485D-A402-82BED62E4A97}"/>
-    <hyperlink ref="F57" r:id="rId43" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2025/63/630/lei-ordinaria-n-630-2025-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{64BC75ED-1964-4204-BAFA-49F3A4083336}"/>
-    <hyperlink ref="F58" r:id="rId44" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2024/62/614/lei-ordinaria-n-614-2024-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{0661ED8C-7E04-4235-BDA6-165CAA2FD04B}"/>
-    <hyperlink ref="F59" r:id="rId45" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2023/59/588/lei-ordinaria-n-588-2023-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{4A341ABB-8BE7-4A6E-B4C1-532DBB4378D2}"/>
-    <hyperlink ref="F61" r:id="rId46" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2021/54/534/lei-ordinaria-n-534-2021-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{95B75048-0C9A-47CB-8A73-3D8052953EA1}"/>
-    <hyperlink ref="F62" r:id="rId47" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2020/52/516/lei-ordinaria-n-516-2020-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{46529EB6-AC15-4D01-B558-28DB00531128}"/>
-    <hyperlink ref="F64" r:id="rId48" xr:uid="{EE42FF6B-39FA-43BE-8F7C-A56762A03BE5}"/>
-    <hyperlink ref="F65" r:id="rId49" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2024/232/2320/lei-ordinaria-n-2320-2024-autoriza-revisao-geral-da-remuneracao-e-os-subsidios-dos-servidores-publicos-e-agentes-politicos-dos-poderes-executivo-e-legislativo-do-municipio-nos-termos-do-artigo-7-caput-iv-e-o-do-artigo-39-3-da-constituicao-federal-extensivo-aos-conselheiros-tutelares-e-aos-proventos-dos-inativos-e-pensionistas?q=Revis%C3%A3o+geraL" xr:uid="{4F7B275E-5955-4B1B-94E6-A35B6D80FEE2}"/>
-    <hyperlink ref="F69" r:id="rId50" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2021/218/2180/lei-ordinaria-n-2180-2021-suspende-os-efeitos-da-lei-municipal-n-2147-2021-que-autoriza-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-e-da-outras-providencias?q=Revis%E3o%20geraL" xr:uid="{EB57F7DB-CDEF-4A7C-9E25-23B1204FA785}"/>
-    <hyperlink ref="F70" r:id="rId51" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2020/211/2107/lei-ordinaria-n-2107-2020-autoriza-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-a-aplicacao-do-artigo-7-inciso-iv-e-art-39-3-da-constituicao-federal-a-remuneracao-dos-servidores-publicos-o-reajuste-dos-proventos-dos-inativos-e-pensionistas-a-recomposicao-dos-subsidios-dos-agentes-politicos-e-fixa-os-pisos-nacionais-minimos-para-os-integrantes-do-magisterio-municipal-11739-2008-e-da-outras-providencias?q=Revis%E3o%20geraL" xr:uid="{924B3E23-6A28-4DA7-BF55-853A35BD0084}"/>
-    <hyperlink ref="F67" r:id="rId52" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2021/220/2198/lei-ordinaria-n-2198-2021-autoriza-revisao-geral-da-remuneracao-dos-servidores-publicos-autoriza-a-aplicacao-do-artigo-7-caput-iv-e-o-do-artigo-39-3-da-constituicao-federal-a-remuneracao-dos-servidores-publicos-e-autoriza-o-reajuste-dos-proventos-dos-inativos-e-pensionistas?q=2.198" xr:uid="{D3688214-1F73-4C24-86E5-7E744B395889}"/>
-    <hyperlink ref="F68" r:id="rId53" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2021/220/2197/lei-ordinaria-n-2197-2021-autoriza-revisao-geral-da-remuneracao-dos-servidores-publicos-autoriza-a-aplicacao-do-artigo-7-caput-iv-e-o-do-artigo-39-3-da-constituicao-federal-a-remuneracao-dos-servidores-publicos-e-autoriza-o-reajuste-dos-proventos-dos-inativos-e-pensionistas?q=2.197" xr:uid="{824C9DCD-78D8-43FD-8DB5-0E165BC5D312}"/>
-    <hyperlink ref="F66" r:id="rId54" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2023/226/2251/lei-ordinaria-n-2251-2023-autoriza-revisao-geral-da-remuneracao-e-os-subsidios-dos-servidores-publicos-e-agentes-politicos-dos-poderes-executivo-e-legislativo-do-municipio-nos-termos-do-artigo-7-caput-iv-e-o-do-artigo-39-3-da-constituicao-federal-extensivo-aos-conselheiros-tutelares-e-aos-proventos-dos-inativos-e-pensionistas?q=Autoriza%20revis%E3o%20geral%20da%20remunera%E7%E3o" xr:uid="{7E99F84F-40DA-489D-BFB8-FC337539CA92}"/>
-    <hyperlink ref="F27" r:id="rId55" xr:uid="{6761F2DF-2A70-4664-8013-B14C436BF884}"/>
+    <hyperlink ref="F37" r:id="rId24" xr:uid="{0198FF07-6ABC-4FE0-BC94-9626A092EF1E}"/>
+    <hyperlink ref="F38" r:id="rId25" xr:uid="{9B9DADFC-147D-439F-A89B-8D7EC2EFFA45}"/>
+    <hyperlink ref="F39" r:id="rId26" xr:uid="{7B4312A5-B4D6-48C3-9967-D4A547A0F189}"/>
+    <hyperlink ref="F43" r:id="rId27" xr:uid="{B555F1DF-7AE0-4CE3-A746-A72DB71A3814}"/>
+    <hyperlink ref="F46" r:id="rId28" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2025/1/3/lei-ordinaria-n-3-2025-concede-recomposicao-e-reajuste-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{79AF655C-919A-4B59-8D63-6E9B71A0DFD8}"/>
+    <hyperlink ref="F47" r:id="rId29" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2024/1/6/lei-ordinaria-n-6-2024-concede-recomposicao-e-reajuste-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-e-recomposicao-inflacionaria-aos-agentes-politicos-do-poder-executivo-prefeito-vice-prefeito-e-secretarios-municipais-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{28DF2AEC-02FD-4904-92E4-8F1A46B7C53A}"/>
+    <hyperlink ref="F48" r:id="rId30" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2023/1/3/lei-ordinaria-n-3-2023-concede-recomposicao-e-reajuste-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-e-recomposicao-inflacionaria-aos-agentes-politicos-do-poder-executivo-prefeito-vice-prefeito-e-secretarios-municipais-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{D52BDBF7-13A5-4A80-A127-116B587657FB}"/>
+    <hyperlink ref="F49" r:id="rId31" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2022/1/5/lei-ordinaria-n-5-2022-concede-recomposicao-e-reajuste-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{3E75ABFE-1194-4B2F-AF68-D20DEC412ED8}"/>
+    <hyperlink ref="F50" r:id="rId32" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2021/1/5/lei-ordinaria-n-5-2021-concede-recomposicao-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-desta-municipalidade-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{4FC8FEEE-0401-4369-8921-ED4B51F5562D}"/>
+    <hyperlink ref="F51" r:id="rId33" display="https://leismunicipais.com.br/a/pr/j/jaguapita/lei-ordinaria/2020/2/11/lei-ordinaria-n-11-2020-concede-recomposicao-salarial-aos-servidores-da-administracao-direta-e-indireta-do-poder-executivo-e-ao-prefeito-vice-prefeito-e-secretarios-municipais-desta-municipalidade-nos-termos-do-artigo-37-x-da-constituicao-federal-e-da-outras-providencias?q=recomposi%E7%E3o%20salarial" xr:uid="{4D8E764E-22B9-4B1F-A195-598C7E088B03}"/>
+    <hyperlink ref="F56" r:id="rId34" xr:uid="{469628B4-8B6D-46C9-A62E-832B5D06C62E}"/>
+    <hyperlink ref="F59" r:id="rId35" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2020/74/739/lei-ordinaria-n-739-2020-dispoe-sobre-a-revisao-geral-anual-do-subsidio-do-prefeito-vice-prefeito-vereadores-secretarios-as-municipais-e-remuneracao-do-s-servidor-es-comissionados-e-estatutario-do-poder-legislativo-do-municipio-de-primeiro-de-maio-e-da-outras-providencias?q=salarial%20" xr:uid="{8F367E47-ABB7-4AAB-A611-4BB40BDA61A3}"/>
+    <hyperlink ref="F54" r:id="rId36" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2025/97/970/lei-ordinaria-n-970-2025-dispoe-sobre-a-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-municipais-de-primeiro-de-maio-e-da-outras-providencias?q=revis%E3o%20geral%20anual%20" xr:uid="{9C1E9D0B-D3E4-4ECB-928C-3AB9384788C0}"/>
+    <hyperlink ref="F55" r:id="rId37" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2024/94/934/lei-ordinaria-n-934-2024-dispoe-sobre-a-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-municipais-de-primeiro-de-maio-e-da-outras-providencias?q=revis%E3o%20geral%20anual%20" xr:uid="{AF964D4D-7701-48C8-898F-A6225D73AC79}"/>
+    <hyperlink ref="F57" r:id="rId38" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2022/80/800/lei-ordinaria-n-800-2022-dispoe-sobre-a-revisao-geral-anual-do-subsidio-do-prefeito-vice-prefeito-vereadores-secretarios-as-municipais-e-remuneracao-do-s-servidor-es-comissionados-e-estatutario-do-poder-legislativo-do-municipio-de-primeiro-de-maio-e-da-outras-providencias?q=revis%E3o%20geral%20anual%20" xr:uid="{98F545B3-8D3D-44B1-AB35-4AC2759963EB}"/>
+    <hyperlink ref="F58" r:id="rId39" display="https://leismunicipais.com.br/a/pr/p/primeiro-de-maio/lei-ordinaria/2021/77/770/lei-ordinaria-n-770-2021-dispoe-sobre-a-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-municipais-de-primeiro-de-maio-e-da-outras-providencias?q=revis%E3o%20geral%20anual%20" xr:uid="{C52DDB23-FB88-489B-BD74-E79A0801ADF5}"/>
+    <hyperlink ref="F41" r:id="rId40" xr:uid="{878A7E66-55B4-4DAF-8A75-A1CF624BBEC7}"/>
+    <hyperlink ref="F40" r:id="rId41" xr:uid="{47F34AB3-0A0A-412F-8FE1-03EF5CACC9CA}"/>
+    <hyperlink ref="F65" r:id="rId42" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-complementar/2022/59/583/lei-complementar-n-583-2022-dispoe-sobre-aumento-salarial-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=aumento%20salarial" xr:uid="{9456DAAA-0A8A-485D-A402-82BED62E4A97}"/>
+    <hyperlink ref="F62" r:id="rId43" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2025/63/630/lei-ordinaria-n-630-2025-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{64BC75ED-1964-4204-BAFA-49F3A4083336}"/>
+    <hyperlink ref="F63" r:id="rId44" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2024/62/614/lei-ordinaria-n-614-2024-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{0661ED8C-7E04-4235-BDA6-165CAA2FD04B}"/>
+    <hyperlink ref="F64" r:id="rId45" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2023/59/588/lei-ordinaria-n-588-2023-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{4A341ABB-8BE7-4A6E-B4C1-532DBB4378D2}"/>
+    <hyperlink ref="F66" r:id="rId46" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2021/54/534/lei-ordinaria-n-534-2021-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{95B75048-0C9A-47CB-8A73-3D8052953EA1}"/>
+    <hyperlink ref="F67" r:id="rId47" display="https://leismunicipais.com.br/a2/pr/p/prado-ferreira/lei-ordinaria/2020/52/516/lei-ordinaria-n-516-2020-dispoe-sobre-a-reposicao-de-perdas-salariais-dos-servidores-publicos-do-municipio-de-prado-ferreira-estado-do-parana-e-da-outras-providencias?q=salarial" xr:uid="{46529EB6-AC15-4D01-B558-28DB00531128}"/>
+    <hyperlink ref="F70" r:id="rId48" xr:uid="{EE42FF6B-39FA-43BE-8F7C-A56762A03BE5}"/>
+    <hyperlink ref="F71" r:id="rId49" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2024/232/2320/lei-ordinaria-n-2320-2024-autoriza-revisao-geral-da-remuneracao-e-os-subsidios-dos-servidores-publicos-e-agentes-politicos-dos-poderes-executivo-e-legislativo-do-municipio-nos-termos-do-artigo-7-caput-iv-e-o-do-artigo-39-3-da-constituicao-federal-extensivo-aos-conselheiros-tutelares-e-aos-proventos-dos-inativos-e-pensionistas?q=Revis%C3%A3o+geraL" xr:uid="{4F7B275E-5955-4B1B-94E6-A35B6D80FEE2}"/>
+    <hyperlink ref="F75" r:id="rId50" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2021/218/2180/lei-ordinaria-n-2180-2021-suspende-os-efeitos-da-lei-municipal-n-2147-2021-que-autoriza-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-e-da-outras-providencias?q=Revis%E3o%20geraL" xr:uid="{EB57F7DB-CDEF-4A7C-9E25-23B1204FA785}"/>
+    <hyperlink ref="F76" r:id="rId51" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2020/211/2107/lei-ordinaria-n-2107-2020-autoriza-revisao-geral-anual-da-remuneracao-dos-servidores-publicos-a-aplicacao-do-artigo-7-inciso-iv-e-art-39-3-da-constituicao-federal-a-remuneracao-dos-servidores-publicos-o-reajuste-dos-proventos-dos-inativos-e-pensionistas-a-recomposicao-dos-subsidios-dos-agentes-politicos-e-fixa-os-pisos-nacionais-minimos-para-os-integrantes-do-magisterio-municipal-11739-2008-e-da-outras-providencias?q=Revis%E3o%20geraL" xr:uid="{924B3E23-6A28-4DA7-BF55-853A35BD0084}"/>
+    <hyperlink ref="F73" r:id="rId52" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2021/220/2198/lei-ordinaria-n-2198-2021-autoriza-revisao-geral-da-remuneracao-dos-servidores-publicos-autoriza-a-aplicacao-do-artigo-7-caput-iv-e-o-do-artigo-39-3-da-constituicao-federal-a-remuneracao-dos-servidores-publicos-e-autoriza-o-reajuste-dos-proventos-dos-inativos-e-pensionistas?q=2.198" xr:uid="{D3688214-1F73-4C24-86E5-7E744B395889}"/>
+    <hyperlink ref="F74" r:id="rId53" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2021/220/2197/lei-ordinaria-n-2197-2021-autoriza-revisao-geral-da-remuneracao-dos-servidores-publicos-autoriza-a-aplicacao-do-artigo-7-caput-iv-e-o-do-artigo-39-3-da-constituicao-federal-a-remuneracao-dos-servidores-publicos-e-autoriza-o-reajuste-dos-proventos-dos-inativos-e-pensionistas?q=2.197" xr:uid="{824C9DCD-78D8-43FD-8DB5-0E165BC5D312}"/>
+    <hyperlink ref="F72" r:id="rId54" display="https://leismunicipais.com.br/a/pr/s/santa-fe/lei-ordinaria/2023/226/2251/lei-ordinaria-n-2251-2023-autoriza-revisao-geral-da-remuneracao-e-os-subsidios-dos-servidores-publicos-e-agentes-politicos-dos-poderes-executivo-e-legislativo-do-municipio-nos-termos-do-artigo-7-caput-iv-e-o-do-artigo-39-3-da-constituicao-federal-extensivo-aos-conselheiros-tutelares-e-aos-proventos-dos-inativos-e-pensionistas?q=Autoriza%20revis%E3o%20geral%20da%20remunera%E7%E3o" xr:uid="{7E99F84F-40DA-489D-BFB8-FC337539CA92}"/>
+    <hyperlink ref="F28" r:id="rId55" xr:uid="{6761F2DF-2A70-4664-8013-B14C436BF884}"/>
+    <hyperlink ref="F20" r:id="rId56" display="https://leismunicipais.com.br/a/pr/c/cafeara/lei-ordinaria/2026/70/698/lei-ordinaria-n-698-2026-autoriza-o-executivo-municipal-a-conceder-recomposicao-geral-anual-aos-servidores-publicos-municipais-e-aos-agentes-politicos-do-poder-executivo-municipal-de-cafeara-e-da-outras-providencias?q=698" xr:uid="{5404D9FC-CD11-4D4E-85B2-924C2C07E479}"/>
+    <hyperlink ref="F69" r:id="rId57" display="https://leis.org/municipais/pr/santa-fe/lei/lei-ordinaria/2026/2453/lei-ordinaria-n-2453-2026-autoriza-revisao-geral-da-remuneracao-dos-servidores-publicos-dos-poderes-executivo-e-legislativo-do-municipio-nos-termos-do-artigo-7-caput-iv-e-do-artigo-39-3-da-constituicao-federal-extensivo-aos-proventos-dos-inativos-e-pensionistas" xr:uid="{D77F6506-3111-4AA7-9B32-D69A2F20804F}"/>
+    <hyperlink ref="F61" r:id="rId58" xr:uid="{97423D6D-B160-4C4A-8E55-34C9690DB996}"/>
+    <hyperlink ref="F53" r:id="rId59" xr:uid="{6D2BAB16-9897-4B5E-8FF2-A635F482C418}"/>
+    <hyperlink ref="F36" r:id="rId60" xr:uid="{B2A96C0D-7BBD-4F5C-B8B2-7F050AFBC606}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId56"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId61"/>
 </worksheet>
 </file>
 
@@ -2416,4 +2588,34 @@
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5740BF14-BE3A-4302-AEE6-B60DD35AC8AB}">
+  <dimension ref="F5:F10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="6:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="F5" s="17">
+        <v>6.3700000000000007E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="6:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="F6" s="17">
+        <v>3.6299999999999999E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F10" s="18">
+        <f>SUM(F3:F7)</f>
+        <v>0.1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>